<commit_message>
Correct GSLERP entry: no open call, and guard against archived calls
GSLERP was listed as an open rolling EOI. It is not. The GCF approved the
project in 2020 for a seven-year run and it is now in delivery with 17 NGO
implementing partners and 5 seedling suppliers already engaged; the call for
proposals is an undated archived page on an aggregator site. Reframed as a
relationship target (Global Shea Alliance membership and the GSA private-sector
members funding the PPPs) with no application route.

Adds a research rule to the skill requiring proof that a call is live before
listing it as open - a future deadline, a dated page on the funder's own domain,
or current-cycle language - and requiring an active check for signs the window
closed, such as named partners already selected or a project in mid-delivery.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PULTYHtQSMT98yhFaxzQDo
</commit_message>
<xml_diff>
--- a/Give-to-Africa-Grant-Pipeline-2026.xlsx
+++ b/Give-to-Africa-Grant-Pipeline-2026.xlsx
@@ -1448,7 +1448,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>UNDP / Green Climate Fund - Ghana Shea Landscape Emission Reductions Project (GSLERP) - NGO partnership pathway</t>
+          <t>UNDP / Green Climate Fund - Ghana Shea Landscape Emission Reductions Project (GSLERP) - RELATIONSHIP ONLY, no open call</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1458,32 +1458,32 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>OPEN - partnership pathway via Expression of Interest</t>
+          <t>NO OPEN CALL - implementing partners already selected</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Project total $54.5M ($30.1M GCF grant, ~$15M Government of Ghana, ~$9M private investment). Individual partner awards not published.</t>
+          <t>Project total $54.5M. No open partner award - the 17 NGO implementing partner slots are filled.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Rolling Expression of Interest to the Global Shea Alliance</t>
+          <t>No open call. The NGO call for proposals is archived - it dates from the project's 2020-21 startup.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>rolling</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>NGOs in Ghana with experience in agroforestry, parkland management and knowledge of the northern savannah zone. Two stages: submit an EOI to the Global Shea Alliance, then pair with a private sector partner in a PPP. Applications MUST include women's cooperatives who will manage community nurseries.</t>
+          <t>NOT CURRENTLY OPEN. The original two-stage EOI (NGO submits to Global Shea Alliance, then pairs with a GSA private-sector member in a PPP including women's cooperatives) ran during project startup. GSLERP was approved by the GCF in 2020 for a seven-year run and is now in delivery with 17 NGO implementing partners and 5 seedling suppliers already engaged.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>NEAR-PERFECT fit. Same geography (Northern Savannah Zone), same commodity (shea), same beneficiaries (women's cooperatives), same climate framing. The project already supports 26 women's cooperatives and explicitly seeks NGO partners. This is the closest thing on the list to a program written for the MDF Ghana partnership.</t>
+          <t>Thematically the closest match found - Northern Savannah Zone, shea, women's cooperatives, climate. But there is no application route, so it is a relationship target, not a funding opportunity. The live angle is the surrounding ecosystem: Global Shea Alliance membership, the private-sector GSA members who co-fund PPPs, and the W+ Standard work GSLERP began in 2025 to quantify women's outcomes.</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1508,12 +1508,12 @@
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
-          <t>HIGHEST-VALUE ACTION ON THIS LIST. Contact the Global Shea Alliance about the EOI process and confirm whether the window is still open. Give to Africa already has the women's cooperative relationships GSLERP requires - that is the scarce ingredient, not the paperwork.</t>
+          <t>Do NOT look for an application portal - there isn't one. Instead join / engage the Global Shea Alliance as a member and get known to the GSA private-sector companies funding the PPPs. Ask GSA directly whether partner intake will reopen before the project closes (~2027) and what a successor project looks like. The W+ Standard adoption is also worth tracking - it is a credential Give to Africa's cooperatives could carry.</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>Project structure, partners, funding split and two-stage EOI process confirmed via UNDP; current EOI window status NOT confirmed</t>
+          <t>CORRECTED Jul 29, 2026. Previously listed as an open rolling EOI - that was wrong. The call for proposals is an undated archived page; project timeline (2020 approval, 7 years) and the 17 already-selected implementing partners confirm the window closed years ago.</t>
         </is>
       </c>
       <c r="P13" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Flag GFCF eligibility risk for a US-registered applicant
GFCF's geographic preference is for organizations based in the Global South, and
the Global North exception is written for orgs serving disadvantaged communities
within the Global North - not a US intermediary regranting into Africa. GFCF also
leads #ShiftThePower, whose premise is reducing Northern intermediaries. Records
the risk and the two better routes rather than leaving it as an unqualified
best-fit recommendation.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PULTYHtQSMT98yhFaxzQDo
</commit_message>
<xml_diff>
--- a/Give-to-Africa-Grant-Pipeline-2026.xlsx
+++ b/Give-to-Africa-Grant-Pipeline-2026.xlsx
@@ -1116,7 +1116,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>OPEN - rolling, no deadline</t>
+          <t>OPEN - rolling, but eligibility needs resolving first</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -1136,12 +1136,12 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Community philanthropy organizations based in Africa, Asia, Middle East, CEE, or Latin America - including national public foundations, women's funds, and grassroots grantmakers. Two-stage process: concept note first, full application by invitation.</t>
+          <t>Community philanthropy organizations, community foundations, women's funds, environmental funds, national public foundations and grassroots grantmakers. GEOGRAPHIC PREFERENCE is for organizations BASED IN Sub-Saharan Africa, MENA, East Asia Pacific, Eastern Europe/Central Asia, and Latin America - regions with limited access to funding. Global North applicants are considered only case-by-case, and that exception is written for organizations serving disadvantaged communities WITHIN the Global North.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>STRONGEST fit on this list for YENDAA and Fiscal Sponsorship. GFCF funds exactly the thing Give to Africa is building - infrastructure that moves resources to locally led African organizations. The 'philanthropy, technology and innovation' positioning line was written for this funder.</t>
+          <t>Programmatically the best mission match on the list - GFCF funds exactly the local-resource-mobilization infrastructure YENDAA and the fiscal sponsorship program represent. BUT there is a structural eligibility risk: Give to Africa is a San Diego-registered 501(c)(3), and GFCF leads the #ShiftThePower movement, whose explicit premise is reducing the role of Northern intermediaries between donors and Global South communities. A US-headquartered org applying to regrant into Africa runs against that thesis. The strong version of this application has an AFRICA-REGISTERED entity as the applicant.</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1171,12 +1171,12 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>Submit a concept note within the next 2 weeks. Lead with YENDAA as African-led giving infrastructure and the November fiscal-sponsorship cohort as proof of local-resource mobilization. Small dollar amount, but it opens a door to a network of community philanthropy funders.</t>
+          <t>Do NOT write the full concept note as Give to Africa (San Diego) without resolving eligibility first. Two better routes: (a) have an Africa-registered partner apply as the lead - MDF Ghana or a fiscal sponsorship cohort member - with Give to Africa named as a supporting partner; or (b) send a short eligibility query to info@globalfundcf.org describing the structure before investing writing time. Check https://globalfundcommunityfoundations.org/what-we-do/grants/who-can-apply/ first.</t>
         </is>
       </c>
       <c r="P8" s="4" t="inlineStr">
         <is>
-          <t>Grant range, rolling process and email confirmed. CORRECTED Jul 29, 2026: the website was previously listed as globalfundcf.org - the live site is globalfundcommunityfoundations.org (the short domain is used for email only).</t>
+          <t>Grant range, rolling process, funding tracks and eligible activities confirmed from GFCF's own site. ELIGIBILITY RISK ADDED Jul 29, 2026: geographic preference is for organizations based in the Global South; the Global North exception is for orgs serving disadvantaged communities within the Global North, which is not Give to Africa's profile. Not a confirmed disqualification - confirm with GFCF.</t>
         </is>
       </c>
       <c r="Q8" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Record GFCF's confirmed eligibility criteria from their own page
Replaces the summarized eligibility with the full four-group self-assessment.
Confirms Give to Africa fails the 'based in' question and is weak on serving a
defined community and building local giving within it - a stretch rather than an
automatic disqualification, since the test is 'yes to most'.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PULTYHtQSMT98yhFaxzQDo
</commit_message>
<xml_diff>
--- a/Give-to-Africa-Grant-Pipeline-2026.xlsx
+++ b/Give-to-Africa-Grant-Pipeline-2026.xlsx
@@ -1136,7 +1136,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Community philanthropy organizations, community foundations, women's funds, environmental funds, national public foundations and grassroots grantmakers. GEOGRAPHIC PREFERENCE is for organizations BASED IN Sub-Saharan Africa, MENA, East Asia Pacific, Eastern Europe/Central Asia, and Latin America - regions with limited access to funding. Global North applicants are considered only case-by-case, and that exception is written for organizations serving disadvantaged communities WITHIN the Global North.</t>
+          <t>Self-assessment against ~15 questions in four groups; GFCF says apply if 'yes' to MOST. (1) ORG TYPE: community philanthropy org, community foundation, women's fund, environmental fund, national public foundation, grassroots grantmaker, OR any other org that identifies with community philanthropy practice - that last catch-all is the widest door. (2) INTEREST IN: shifting power closer to communities; growing LOCAL assets as a central pillar; piloting new governance / decision-making / local resource mobilization approaches. (3) DOES YOUR ORG: serve a particular community (geographic, issue or identity based); use grantmaking to devolve power and resources; build a LOCAL culture of giving WITHIN the community you serve; build trust and networks; take on complex or unpopular issues. (4) BASED IN: Africa, Asia, Middle East, CEE, or Latin America &amp; Caribbean - priority where other funding is scarce. Global North applicants considered case-by-case, but that exception is framed for orgs REPRESENTING DISADVANTAGED COMMUNITIES IN THE GLOBAL NORTH.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="P8" s="4" t="inlineStr">
         <is>
-          <t>Grant range, rolling process, funding tracks and eligible activities confirmed from GFCF's own site. ELIGIBILITY RISK ADDED Jul 29, 2026: geographic preference is for organizations based in the Global South; the Global North exception is for orgs serving disadvantaged communities within the Global North, which is not Give to Africa's profile. Not a confirmed disqualification - confirm with GFCF.</t>
+          <t>Full eligibility criteria confirmed Jul 29, 2026 from GFCF's own 'Who can apply' page. Give to Africa fails the 'based in' question outright (San Diego) and is weak on 'serve a particular community' and 'build a LOCAL culture of giving within the community you serve'. Not an automatic disqualification - the test is 'yes to most' - but a US-led application is a stretch.</t>
         </is>
       </c>
       <c r="Q8" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Correct MDF: Minerals Development Fund is a Ghanaian statutory public fund
MDF was recorded as if it were an NGO implementing partner. It is the Minerals
Development Fund (mdf.gov.gh), established by Act 912 of 2016 under the Ministry
of Lands and Natural Resources and capitalised by 20% of national mineral
royalties to fund development in mining-affected communities. That government
institutional status is a materially stronger credential than a partner mention,
and the context file now says so explicitly.

Also records Sunyani Technical University and University of Cincinnati as design
partners, and the facility's solar processing and community water scope.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PULTYHtQSMT98yhFaxzQDo
</commit_message>
<xml_diff>
--- a/Give-to-Africa-Grant-Pipeline-2026.xlsx
+++ b/Give-to-Africa-Grant-Pipeline-2026.xlsx
@@ -592,7 +592,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Give to Africa - Grant Pipeline (Government, Multilateral &amp; Foundation)  |  Last updated July 29, 2026  |  23 opportunities tracked</t>
+          <t>Give to Africa - Grant Pipeline (Government, Multilateral &amp; Foundation)  |  Last updated July 30, 2026  |  23 opportunities tracked</t>
         </is>
       </c>
     </row>
@@ -804,12 +804,12 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Agribusinesses, cooperatives and agritech firms operating in Sub-Saharan Africa / South Asia with proven smallholder-farmer linkages. Likely needs MDF Ghana or a shea cooperative as the applicant entity, with Give to Africa as technical/fiscal partner.</t>
+          <t>Agribusinesses, cooperatives and agritech firms operating in Sub-Saharan Africa / South Asia with proven smallholder-farmer linkages. Likely needs the Minerals Development Fund (MDF), Ghana or a shea cooperative as the applicant entity, with Give to Africa as technical/fiscal partner.</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Climate Resilience Program / MDF Ghana shea butter factories. Eligible uses reportedly include equipment and technology procurement, capacity building, and climate/ESG-aligned investment - which maps onto both the factory build-out and the PPE procurement push.</t>
+          <t>Climate Resilience Program / the Minerals Development Fund (MDF), Ghana shea butter factories. Eligible uses reportedly include equipment and technology procurement, capacity building, and climate/ESG-aligned investment - which maps onto both the factory build-out and the PPE procurement push.</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Strong strategic fit as a corporate partner rather than a funder. The program already funds shelling machines, sustainable parkland training and borehole regeneration for 10,500+ shea collectors - directly adjacent to the MDF Ghana factories and the PPE procurement push.</t>
+          <t>Strong strategic fit as a corporate partner rather than a funder. The program already funds shelling machines, sustainable parkland training and borehole regeneration for 10,500+ shea collectors - directly adjacent to the the Minerals Development Fund (MDF), Ghana factories and the PPE procurement push.</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>Do NOT write the full concept note as Give to Africa (San Diego) without resolving eligibility first. Two better routes: (a) have an Africa-registered partner apply as the lead - MDF Ghana or a fiscal sponsorship cohort member - with Give to Africa named as a supporting partner; or (b) send a short eligibility query to info@globalfundcf.org describing the structure before investing writing time. Check https://globalfundcommunityfoundations.org/what-we-do/grants/who-can-apply/ first.</t>
+          <t>Do NOT write the full concept note as Give to Africa (San Diego) without resolving eligibility first. Two better routes: (a) have an Africa-registered partner apply as the lead - the Minerals Development Fund (MDF), Ghana or a fiscal sponsorship cohort member - with Give to Africa named as a supporting partner; or (b) send a short eligibility query to info@globalfundcf.org describing the structure before investing writing time. Check https://globalfundcommunityfoundations.org/what-we-do/grants/who-can-apply/ first.</t>
         </is>
       </c>
       <c r="P8" s="4" t="inlineStr">
@@ -1219,12 +1219,12 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Applicant must be a non-profit, NGO or CBO registered with the Government of Ghana, or a community association formed at least a year before applying. Give to Africa cannot apply directly - MDF Ghana or a shea cooperative must be the applicant. Requires substantial community contribution (labor, materials, land, expertise).</t>
+          <t>Applicant must be a non-profit, NGO or CBO registered with the Government of Ghana, or a community association formed at least a year before applying. Give to Africa cannot apply directly - the Minerals Development Fund (MDF), Ghana or a shea cooperative must be the applicant. Requires substantial community contribution (labor, materials, land, expertise).</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Climate Resilience / MDF Ghana. A 12-month, community-led shea processing or PPE project is precisely the profile ASSH funds, and the required community contribution is already covered by the existing 80/20 split and 4-to-1 government match.</t>
+          <t>Climate Resilience / the Minerals Development Fund (MDF), Ghana. A 12-month, community-led shea processing or PPE project is precisely the profile ASSH funds, and the required community contribution is already covered by the existing 80/20 split and 4-to-1 government match.</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>PROGRAM PAGE: https://gh.usembassy.gov/education-culture/ambassadors-special-self-help-program/ No live application form is posted between cycles. EMAIL AccraSelfHelp@state.gov to ask for the current Notice of Funding Opportunity and application form. MDF Ghana must be the applicant.</t>
+          <t>PROGRAM PAGE: https://gh.usembassy.gov/education-culture/ambassadors-special-self-help-program/ No live application form is posted between cycles. EMAIL AccraSelfHelp@state.gov to ask for the current Notice of Funding Opportunity and application form. the Minerals Development Fund (MDF), Ghana must be the applicant.</t>
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>Email AccraSelfHelp@state.gov this week asking when the next window opens, and have MDF Ghana ready as the named applicant. Small award, but a U.S. Embassy grant is a credential worth more than $12,000 in later proposals.</t>
+          <t>Email AccraSelfHelp@state.gov this week asking when the next window opens, and have the Minerals Development Fund (MDF), Ghana ready as the named applicant. Small award, but a U.S. Embassy grant is a credential worth more than $12,000 in later proposals.</t>
         </is>
       </c>
       <c r="P9" s="4" t="inlineStr">
@@ -1634,12 +1634,12 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Local Ghanaian NGOs/non-profits with valid Registrar General's Department and Social Welfare certificates, or CBOs / social enterprises recognized by the District Assembly and Ghana EPA. MDF Ghana would be the applicant; Give to Africa cannot apply directly.</t>
+          <t>Local Ghanaian NGOs/non-profits with valid Registrar General's Department and Social Welfare certificates, or CBOs / social enterprises recognized by the District Assembly and Ghana EPA. the Minerals Development Fund (MDF), Ghana would be the applicant; Give to Africa cannot apply directly.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>EXCELLENT strategic fit. The 2026 priority geography was the Black Volta Basin - Wa-West (Upper West), Bole, Sawla-Tuna-Kalba and Central Gonja (Savannah Region) - which is the same northern Ghana shea-gathering belt the MDF Ghana partnership already works in. Focus areas include sustainable agriculture and community-based conservation.</t>
+          <t>EXCELLENT strategic fit. The 2026 priority geography was the Black Volta Basin - Wa-West (Upper West), Bole, Sawla-Tuna-Kalba and Central Gonja (Savannah Region) - which is the same northern Ghana shea-gathering belt the the Minerals Development Fund (MDF), Ghana partnership already works in. Focus areas include sustainable agriculture and community-based conservation.</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1659,7 +1659,7 @@
       </c>
       <c r="M14" s="7" t="inlineStr">
         <is>
-          <t>NO OPEN CALL - the 2026 round closed Mar 13. Calls are posted on the UNDP Ghana site and the country page at https://sgp.undp.org (Ghana). CONTACT: the 2026 call published akosua.bireduaa.aninakwa@undp.org for enquiries - email to confirm the 2027 timetable. MDF Ghana must be the applicant and needs valid Registrar General + Social Welfare certificates.</t>
+          <t>NO OPEN CALL - the 2026 round closed Mar 13. Calls are posted on the UNDP Ghana site and the country page at https://sgp.undp.org (Ghana). CONTACT: the 2026 call published akosua.bireduaa.aninakwa@undp.org for enquiries - email to confirm the 2027 timetable. the Minerals Development Fund (MDF), Ghana must be the applicant and needs valid Registrar General + Social Welfare certificates.</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>Put a calendar reminder for early February 2027. Confirm now that MDF Ghana's Registrar General and Social Welfare certificates are current - that paperwork is the usual disqualifier, and it takes months to fix.</t>
+          <t>Put a calendar reminder for early February 2027. Confirm now that the Minerals Development Fund (MDF), Ghana's Registrar General and Social Welfare certificates are current - that paperwork is the usual disqualifier, and it takes months to fix.</t>
         </is>
       </c>
       <c r="P14" s="4" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>2026 Ghana themes were democratic governance / human rights and peace &amp; security, with gender equality as a cross-cutting theme. Themes rotate year to year - if a 2027 theme touches women's economic empowerment or climate, the MDF Ghana shea work fits cleanly.</t>
+          <t>2026 Ghana themes were democratic governance / human rights and peace &amp; security, with gender equality as a cross-cutting theme. Themes rotate year to year - if a 2027 theme touches women's economic empowerment or climate, the the Minerals Development Fund (MDF), Ghana shea work fits cleanly.</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1888,7 +1888,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>BEST NEW FIND. The MDF Ghana shea butter factories are a job-creation investment in exactly the country and sector IFE funds, and the 90% cost coverage for non-revenue non-profit projects is unusually generous. Scale is far above anything else on this list.</t>
+          <t>BEST NEW FIND. The the Minerals Development Fund (MDF), Ghana shea butter factories are a job-creation investment in exactly the country and sector IFE funds, and the 90% cost coverage for non-revenue non-profit projects is unusually generous. Scale is far above anything else on this list.</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>Email the CfP address now to ask to be notified when the 2027 window opens and to confirm whether a U.S. 501(c)(3) can apply directly or must partner with MDF Ghana. Start modelling the factory job-creation numbers - that is the metric IFE selects on.</t>
+          <t>Email the CfP address now to ask to be notified when the 2027 window opens and to confirm whether a U.S. 501(c)(3) can apply directly or must partner with the Minerals Development Fund (MDF), Ghana. Start modelling the factory job-creation numbers - that is the metric IFE selects on.</t>
         </is>
       </c>
       <c r="P17" s="4" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>Watch for the 29th call announcement. Before applying, decide whether MDF Ghana's factory model can service debt - if not, this is the wrong instrument regardless of fit.</t>
+          <t>Watch for the 29th call announcement. Before applying, decide whether the Minerals Development Fund (MDF), Ghana's factory model can service debt - if not, this is the wrong instrument regardless of fit.</t>
         </is>
       </c>
       <c r="P18" s="4" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Applicant must be a 100% African-owned enterprise, cooperative, producer group or processor in an eligible country. Give to Africa is NOT directly eligible - the shea cooperative or MDF Ghana would be the grantee, with Give to Africa providing proposal and compliance support.</t>
+          <t>Applicant must be a 100% African-owned enterprise, cooperative, producer group or processor in an eligible country. Give to Africa is NOT directly eligible - the shea cooperative or the Minerals Development Fund (MDF), Ghana would be the grantee, with Give to Africa providing proposal and compliance support.</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add three private/corporate foundation leads
- Conservation, Food and Health Foundation: strongest direct-apply fit found.
  5-50K/year, focus areas map onto the Ghana programme, and eligibility turns
  on where the work happens rather than where the applicant is registered, so
  Give to Africa can apply as itself.
- Draper Richards Kaplan: rolling, YENDAA-shaped, flagged as unverified.
- Smart & Final: recorded as NOT ELIGIBLE. Their giving is restricted to
  communities the company serves in AZ/CA/NV; all four Give to Africa programs
  operate in Africa. Kept so the ground is not re-searched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PULTYHtQSMT98yhFaxzQDo
</commit_message>
<xml_diff>
--- a/Give-to-Africa-Grant-Pipeline-2026.xlsx
+++ b/Give-to-Africa-Grant-Pipeline-2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How to Use + Method" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Grant Pipeline'!$A$2:$Q$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Grant Pipeline'!$A$2:$Q$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -592,7 +592,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Give to Africa - Grant Pipeline (Government, Multilateral &amp; Foundation)  |  Last updated July 30, 2026  |  23 opportunities tracked</t>
+          <t>Give to Africa - Grant Pipeline (Government, Multilateral &amp; Foundation)  |  Last updated July 30, 2026  |  26 opportunities tracked</t>
         </is>
       </c>
     </row>
@@ -1106,27 +1106,27 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Global Fund for Community Foundations (GFCF) - Fostering Community Philanthropy small grants</t>
+          <t>Draper Richards Kaplan Foundation</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Foundation (intermediary funder)</t>
+          <t>Private foundation / venture philanthropy (US)</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>OPEN - rolling, but eligibility needs resolving first</t>
+          <t>OPEN - rolling applications</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>$7,000 - $20,000</t>
+          <t>Reported up to $300,000 over three years</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Rolling - concept notes accepted at any time</t>
+          <t>Rolling</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -1136,22 +1136,22 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Self-assessment against ~15 questions in four groups; GFCF says apply if 'yes' to MOST. (1) ORG TYPE: community philanthropy org, community foundation, women's fund, environmental fund, national public foundation, grassroots grantmaker, OR any other org that identifies with community philanthropy practice - that last catch-all is the widest door. (2) INTEREST IN: shifting power closer to communities; growing LOCAL assets as a central pillar; piloting new governance / decision-making / local resource mobilization approaches. (3) DOES YOUR ORG: serve a particular community (geographic, issue or identity based); use grantmaking to devolve power and resources; build a LOCAL culture of giving WITHIN the community you serve; build trust and networks; take on complex or unpopular issues. (4) BASED IN: Africa, Asia, Middle East, CEE, or Latin America &amp; Caribbean - priority where other funding is scarce. Global North applicants considered case-by-case, but that exception is framed for orgs REPRESENTING DISADVANTAGED COMMUNITIES IN THE GLOBAL NORTH.</t>
+          <t>Early-stage social enterprises and social impact organisations with scalable solutions. Typically funds organisations in their first years, backing the founder as much as the model. Highly competitive.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Programmatically the best mission match on the list - GFCF funds exactly the local-resource-mobilization infrastructure YENDAA and the fiscal sponsorship program represent. BUT there is a structural eligibility risk: Give to Africa is a San Diego-registered 501(c)(3), and GFCF leads the #ShiftThePower movement, whose explicit premise is reducing the role of Northern intermediaries between donors and Global South communities. A US-headquartered org applying to regrant into Africa runs against that thesis. The strong version of this application has an AFRICA-REGISTERED entity as the applicant.</t>
+          <t>YENDAA is the fit here, not the Ghana programme - DRK funds scalable ventures led by a founder, and a digital marketplace for verified African-led causes is the kind of model they back. Give to Africa applies directly as a US 501(c)(3).</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>https://globalfundcommunityfoundations.org</t>
+          <t>https://www.drkfoundation.org</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>info@globalfundcf.org</t>
+          <t>not publicly listed</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
@@ -1159,27 +1159,31 @@
           <t>not publicly listed</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr">
-        <is>
-          <t>APPLY HERE: https://globalfundcommunityfoundations.org/what-we-do/grants/share-a-concept-note/ - an online concept-note form. You can also email the concept note to info@globalfundcf.org. Read their 'who can apply' guidance first: https://globalfundcommunityfoundations.org/what-we-do/grants/our-grantmaking-process-and-approach/ Stage 2 (longer application) is by invitation only.</t>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
+          <t>NO VERIFIED APPLICATION URL CONFIRMED in this search. DRK is reported to accept rolling applications - check drkfoundation.org directly for the current intake process before investing time.</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>https://www2.fundsforngos.org/latest-funds-for-ngos/apply-for-small-grants-to-foster-community-philanthropy/</t>
+          <t>https://www.drkfoundation.org</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>Do NOT write the full concept note as Give to Africa (San Diego) without resolving eligibility first. Two better routes: (a) have an Africa-registered partner apply as the lead - the Minerals Development Fund (MDF), Ghana or a fiscal sponsorship cohort member - with Give to Africa named as a supporting partner; or (b) send a short eligibility query to info@globalfundcf.org describing the structure before investing writing time. Check https://globalfundcommunityfoundations.org/what-we-do/grants/who-can-apply/ first.</t>
-        </is>
-      </c>
-      <c r="P8" s="4" t="inlineStr">
-        <is>
-          <t>Full eligibility criteria confirmed Jul 29, 2026 from GFCF's own 'Who can apply' page. Give to Africa fails the 'based in' question outright (San Diego) and is weak on 'serve a particular community' and 'build a LOCAL culture of giving within the community you serve'. Not an automatic disqualification - the test is 'yes to most' - but a US-led application is a stretch.</t>
-        </is>
-      </c>
-      <c r="Q8" s="4" t="inlineStr"/>
+          <t>Read their portfolio first to judge stage fit honestly - DRK backs a small number of ventures per year and is very selective. Worth a look for YENDAA, but treat as a long shot rather than a pipeline item.</t>
+        </is>
+      </c>
+      <c r="P8" s="8" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION - grant size and rolling process come from aggregator summaries; the funder's own application process was not confirmed.</t>
+        </is>
+      </c>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="96" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
@@ -1189,52 +1193,52 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>U.S. Embassy Ghana - Ambassador's Special Self-Help (ASSH) Program</t>
+          <t>Global Fund for Community Foundations (GFCF) - Fostering Community Philanthropy small grants</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>U.S. Government (embassy small grants)</t>
+          <t>Foundation (intermediary funder)</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>OPEN - annual cycle, confirm current window</t>
+          <t>OPEN - rolling, but eligibility needs resolving first</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>$1,000 - $12,000 (awards typically $2,000 - $10,000)</t>
+          <t>$7,000 - $20,000</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Annual cycle - current 2026 window not published online; email the coordinator to confirm</t>
+          <t>Rolling - concept notes accepted at any time</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rolling</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Applicant must be a non-profit, NGO or CBO registered with the Government of Ghana, or a community association formed at least a year before applying. Give to Africa cannot apply directly - the Minerals Development Fund (MDF), Ghana or a shea cooperative must be the applicant. Requires substantial community contribution (labor, materials, land, expertise).</t>
+          <t>Self-assessment against ~15 questions in four groups; GFCF says apply if 'yes' to MOST. (1) ORG TYPE: community philanthropy org, community foundation, women's fund, environmental fund, national public foundation, grassroots grantmaker, OR any other org that identifies with community philanthropy practice - that last catch-all is the widest door. (2) INTEREST IN: shifting power closer to communities; growing LOCAL assets as a central pillar; piloting new governance / decision-making / local resource mobilization approaches. (3) DOES YOUR ORG: serve a particular community (geographic, issue or identity based); use grantmaking to devolve power and resources; build a LOCAL culture of giving WITHIN the community you serve; build trust and networks; take on complex or unpopular issues. (4) BASED IN: Africa, Asia, Middle East, CEE, or Latin America &amp; Caribbean - priority where other funding is scarce. Global North applicants considered case-by-case, but that exception is framed for orgs REPRESENTING DISADVANTAGED COMMUNITIES IN THE GLOBAL NORTH.</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Climate Resilience / the Minerals Development Fund (MDF), Ghana. A 12-month, community-led shea processing or PPE project is precisely the profile ASSH funds, and the required community contribution is already covered by the existing 80/20 split and 4-to-1 government match.</t>
+          <t>Programmatically the best mission match on the list - GFCF funds exactly the local-resource-mobilization infrastructure YENDAA and the fiscal sponsorship program represent. BUT there is a structural eligibility risk: Give to Africa is a San Diego-registered 501(c)(3), and GFCF leads the #ShiftThePower movement, whose explicit premise is reducing the role of Northern intermediaries between donors and Global South communities. A US-headquartered org applying to regrant into Africa runs against that thesis. The strong version of this application has an AFRICA-REGISTERED entity as the applicant.</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>https://gh.usembassy.gov/ambassadors-special-self-help-program/</t>
+          <t>https://globalfundcommunityfoundations.org</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>AccraSelfHelp@state.gov</t>
+          <t>info@globalfundcf.org</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
@@ -1242,24 +1246,24 @@
           <t>not publicly listed</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
-        <is>
-          <t>PROGRAM PAGE: https://gh.usembassy.gov/education-culture/ambassadors-special-self-help-program/ No live application form is posted between cycles. EMAIL AccraSelfHelp@state.gov to ask for the current Notice of Funding Opportunity and application form. the Minerals Development Fund (MDF), Ghana must be the applicant.</t>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>APPLY HERE: https://globalfundcommunityfoundations.org/what-we-do/grants/share-a-concept-note/ - an online concept-note form. You can also email the concept note to info@globalfundcf.org. Read their 'who can apply' guidance first: https://globalfundcommunityfoundations.org/what-we-do/grants/our-grantmaking-process-and-approach/ Stage 2 (longer application) is by invitation only.</t>
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr">
         <is>
-          <t>https://gh.usembassy.gov/ambassadors-special-self-help-program/</t>
+          <t>https://www2.fundsforngos.org/latest-funds-for-ngos/apply-for-small-grants-to-foster-community-philanthropy/</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>Email AccraSelfHelp@state.gov this week asking when the next window opens, and have the Minerals Development Fund (MDF), Ghana ready as the named applicant. Small award, but a U.S. Embassy grant is a credential worth more than $12,000 in later proposals.</t>
+          <t>Do NOT write the full concept note as Give to Africa (San Diego) without resolving eligibility first. Two better routes: (a) have an Africa-registered partner apply as the lead - the Minerals Development Fund (MDF), Ghana or a fiscal sponsorship cohort member - with Give to Africa named as a supporting partner; or (b) send a short eligibility query to info@globalfundcf.org describing the structure before investing writing time. Check https://globalfundcommunityfoundations.org/what-we-do/grants/who-can-apply/ first.</t>
         </is>
       </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>Amounts and eligibility confirmed; current-cycle deadline NOT confirmed - the embassy page has not published a 2026 date</t>
+          <t>Full eligibility criteria confirmed Jul 29, 2026 from GFCF's own 'Who can apply' page. Give to Africa fails the 'based in' question outright (San Diego) and is weak on 'serve a particular community' and 'build a LOCAL culture of giving within the community you serve'. Not an automatic disqualification - the test is 'yes to most' - but a US-led application is a stretch.</t>
         </is>
       </c>
       <c r="Q9" s="4" t="inlineStr"/>
@@ -1272,7 +1276,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>U.S. Embassy Ghana - Public Diplomacy Section Annual Program Statement (APS)</t>
+          <t>U.S. Embassy Ghana - Ambassador's Special Self-Help (ASSH) Program</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1282,17 +1286,17 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>WATCH - last confirmed cycle closed, reissued annually</t>
+          <t>OPEN - annual cycle, confirm current window</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>$15,000 - $100,000 (range from the most recently confirmed cycle)</t>
+          <t>$1,000 - $12,000 (awards typically $2,000 - $10,000)</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Not currently posted - APS is normally reissued each fiscal year</t>
+          <t>Annual cycle - current 2026 window not published online; email the coordinator to confirm</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1302,22 +1306,22 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Registered non-profits, NGOs, academic institutions and civil society organizations. Two-step: Statement of Interest first, full proposal by invitation. U.S.-based organizations have been eligible in prior Ghana cycles.</t>
+          <t>Applicant must be a non-profit, NGO or CBO registered with the Government of Ghana, or a community association formed at least a year before applying. Give to Africa cannot apply directly - the Minerals Development Fund (MDF), Ghana or a shea cooperative must be the applicant. Requires substantial community contribution (labor, materials, land, expertise).</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Education &amp; Workforce Development - the Bradford University African Philanthropy Studies curriculum is a natural APS project (educational exchange, capacity building, U.S.-Ghana institutional linkage).</t>
+          <t>Climate Resilience / the Minerals Development Fund (MDF), Ghana. A 12-month, community-led shea processing or PPE project is precisely the profile ASSH funds, and the required community contribution is already covered by the existing 80/20 split and 4-to-1 government match.</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>https://gh.usembassy.gov/education-culture/public-affairs-small-grants/</t>
+          <t>https://gh.usembassy.gov/ambassadors-special-self-help-program/</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>PASAccraGrant@state.gov</t>
+          <t>AccraSelfHelp@state.gov</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -1327,22 +1331,22 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>PROGRAM PAGE: https://gh.usembassy.gov/education-culture/public-affairs-small-grants/ No open call posted. EMAIL PASAccraGrant@state.gov to ask when the next Annual Program Statement is issued. When live, step 1 is a short Statement of Interest, not a full proposal.</t>
+          <t>PROGRAM PAGE: https://gh.usembassy.gov/education-culture/ambassadors-special-self-help-program/ No live application form is posted between cycles. EMAIL AccraSelfHelp@state.gov to ask for the current Notice of Funding Opportunity and application form. the Minerals Development Fund (MDF), Ghana must be the applicant.</t>
         </is>
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>https://gh.usembassy.gov/education-culture/public-affairs-small-grants/public-diplomacy-section-annual-program-statement-request-for-statements-of-interest/</t>
+          <t>https://gh.usembassy.gov/ambassadors-special-self-help-program/</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>Email PASAccraGrant@state.gov to ask when the FY2027 APS will be issued and to be added to any notification list. Draft the Bradford curriculum Statement of Interest now so it is ready the day the APS posts.</t>
+          <t>Email AccraSelfHelp@state.gov this week asking when the next window opens, and have the Minerals Development Fund (MDF), Ghana ready as the named applicant. Small award, but a U.S. Embassy grant is a credential worth more than $12,000 in later proposals.</t>
         </is>
       </c>
       <c r="P10" s="4" t="inlineStr">
         <is>
-          <t>Email address and prior-cycle funding range confirmed; no open 2026 call found</t>
+          <t>Amounts and eligibility confirmed; current-cycle deadline NOT confirmed - the embassy page has not published a 2026 date</t>
         </is>
       </c>
       <c r="Q10" s="4" t="inlineStr"/>
@@ -1355,52 +1359,52 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>UK FCDO - Funder Finder / Ghana country office</t>
+          <t>U.S. Embassy Ghana - Public Diplomacy Section Annual Program Statement (APS)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Foreign government (UK)</t>
+          <t>U.S. Government (embassy small grants)</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>MONITORING SOURCE - no Ghana-specific open call identified</t>
+          <t>WATCH - last confirmed cycle closed, reissued annually</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Varies by programme</t>
+          <t>$15,000 - $100,000 (range from the most recently confirmed cycle)</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Varies - Funder Finder is a searchable live database</t>
+          <t>Not currently posted - APS is normally reissued each fiscal year</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>rolling</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Varies by call. FCDO funds CSOs through mechanisms such as Aid Connect, which invites proposals from CSO consortia. Bond advises contacting FCDO country offices directly, as some funding is distributed at country level.</t>
+          <t>Registered non-profits, NGOs, academic institutions and civil society organizations. Two-step: Statement of Interest first, full proposal by invitation. U.S.-based organizations have been eligible in prior Ghana cycles.</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>No open call matched to Give to Africa's programs at the time of this search. Listed as a channel to monitor rather than an opportunity - the Ghana Governance Programme shows FCDO does fund Ghanaian civil society.</t>
+          <t>Education &amp; Workforce Development - the Bradford University African Philanthropy Studies curriculum is a natural APS project (educational exchange, capacity building, U.S.-Ghana institutional linkage).</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>https://devtracker.fcdo.gov.uk/countries/GH/projects/</t>
+          <t>https://gh.usembassy.gov/education-culture/public-affairs-small-grants/</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>not publicly listed</t>
+          <t>PASAccraGrant@state.gov</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
@@ -1408,24 +1412,24 @@
           <t>not publicly listed</t>
         </is>
       </c>
-      <c r="M11" s="7" t="inlineStr">
-        <is>
-          <t>NO SPECIFIC CALL. Search the FCDO Funder Finder and the UK government funding portal for live opportunities, and see Bond's funding page: https://www.bond.org.uk/resources-support/funding/ Bond specifically advises contacting the FCDO Ghana country office directly, since some funds are distributed at country level.</t>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>PROGRAM PAGE: https://gh.usembassy.gov/education-culture/public-affairs-small-grants/ No open call posted. EMAIL PASAccraGrant@state.gov to ask when the next Annual Program Statement is issued. When live, step 1 is a short Statement of Interest, not a full proposal.</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>https://www.bond.org.uk/resources-support/funding/</t>
+          <t>https://gh.usembassy.gov/education-culture/public-affairs-small-grants/public-diplomacy-section-annual-program-statement-request-for-statements-of-interest/</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>Add FCDO Funder Finder to the daily monitor's source rotation. Consider contacting the FCDO Ghana country office directly, which Bond specifically recommends for country-level funds.</t>
+          <t>Email PASAccraGrant@state.gov to ask when the FY2027 APS will be issued and to be added to any notification list. Draft the Bradford curriculum Statement of Interest now so it is ready the day the APS posts.</t>
         </is>
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>Mechanism and guidance confirmed; NO specific open opportunity found</t>
+          <t>Email address and prior-cycle funding range confirmed; no open 2026 call found</t>
         </is>
       </c>
       <c r="Q11" s="4" t="inlineStr"/>
@@ -1438,160 +1442,160 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
+          <t>UK FCDO - Funder Finder / Ghana country office</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Foreign government (UK)</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>MONITORING SOURCE - no Ghana-specific open call identified</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Varies by programme</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Varies - Funder Finder is a searchable live database</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>rolling</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Varies by call. FCDO funds CSOs through mechanisms such as Aid Connect, which invites proposals from CSO consortia. Bond advises contacting FCDO country offices directly, as some funding is distributed at country level.</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>No open call matched to Give to Africa's programs at the time of this search. Listed as a channel to monitor rather than an opportunity - the Ghana Governance Programme shows FCDO does fund Ghanaian civil society.</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>https://devtracker.fcdo.gov.uk/countries/GH/projects/</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>NO SPECIFIC CALL. Search the FCDO Funder Finder and the UK government funding portal for live opportunities, and see Bond's funding page: https://www.bond.org.uk/resources-support/funding/ Bond specifically advises contacting the FCDO Ghana country office directly, since some funds are distributed at country level.</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bond.org.uk/resources-support/funding/</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>Add FCDO Funder Finder to the daily monitor's source rotation. Consider contacting the FCDO Ghana country office directly, which Bond specifically recommends for country-level funds.</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
+          <t>Mechanism and guidance confirmed; NO specific open opportunity found</t>
+        </is>
+      </c>
+      <c r="Q12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13" ht="96" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>2 - Open / rolling</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
           <t>UNDP / Green Climate Fund - Ghana Shea Landscape Emission Reductions Project (GSLERP) - RELATIONSHIP ONLY, no open call</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Multilateral (GCF / UNDP, delivered with the Global Shea Alliance)</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>NO OPEN CALL - implementing partners already selected</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Project total $54.5M. No open partner award - the 17 NGO implementing partner slots are filled.</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>No open call. The NGO call for proposals is archived - it dates from the project's 2020-21 startup.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>NOT CURRENTLY OPEN. The original two-stage EOI (NGO submits to Global Shea Alliance, then pairs with a GSA private-sector member in a PPP including women's cooperatives) ran during project startup. GSLERP was approved by the GCF in 2020 for a seven-year run and is now in delivery with 17 NGO implementing partners and 5 seedling suppliers already engaged.</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Thematically the closest match found - Northern Savannah Zone, shea, women's cooperatives, climate. But there is no application route, so it is a relationship target, not a funding opportunity. The live angle is the surrounding ecosystem: Global Shea Alliance membership, the private-sector GSA members who co-fund PPPs, and the W+ Standard work GSLERP began in 2025 to quantify women's outcomes.</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>https://www.undp.org/ghana/projects/ghana-shea-landscape-emission-reductions-project</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>not publicly listed (EOI is submitted to the Global Shea Alliance - see globalshea.com for contacts)</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M12" s="7" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
         <is>
           <t>NO APPLICATION ROUTE - the call is archived and the 17 implementing partner slots are filled. Do not look for a portal. Engage the Global Shea Alliance (globalshea.com) as a member and ask whether partner intake reopens before the project ends around 2027.</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>https://www.undp.org/ghana/projects/ghana-shea-landscapes-emission-reductions-project-gslerp</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
+      <c r="O13" s="4" t="inlineStr">
         <is>
           <t>Do NOT look for an application portal - there isn't one. Instead join / engage the Global Shea Alliance as a member and get known to the GSA private-sector companies funding the PPPs. Ask GSA directly whether partner intake will reopen before the project closes (~2027) and what a successor project looks like. The W+ Standard adoption is also worth tracking - it is a credential Give to Africa's cooperatives could carry.</t>
         </is>
       </c>
-      <c r="P12" s="8" t="inlineStr">
+      <c r="P13" s="8" t="inlineStr">
         <is>
           <t>CORRECTED Jul 29, 2026. Previously listed as an open rolling EOI - that was wrong. The call for proposals is an undated archived page; project timeline (2020 approval, 7 years) and the 17 already-selected implementing partners confirm the window closed years ago.</t>
-        </is>
-      </c>
-      <c r="Q12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13" ht="96" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>3 - Calendar for next cycle</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>UN Women's Peace &amp; Humanitarian Fund (WPHF) - Rapid Response Window</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Multilateral (UN)</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Not published in the summary reviewed</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Concept notes accepted through Dec 31, 2026</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>International and regional NGOs partnering under the Rapid Response Window, in ODA-eligible countries with active peace processes.</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>WEAK fit. Ghana has no active peace process, so the window's core criterion is not met. Listed only for completeness on the multilateral side.</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>https://wphfund.org</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M13" s="4" t="inlineStr">
-        <is>
-          <t>CALLS ARE POSTED AT: https://wphfund.org - open calls appear there as they launch, each with its own submission instructions. No standing portal. Weak fit for Ghana regardless.</t>
-        </is>
-      </c>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t>https://wphfund.org/call-for-proposals-for-rapid-response-window-i-rngo-partners/</t>
-        </is>
-      </c>
-      <c r="O13" s="4" t="inlineStr">
-        <is>
-          <t>Deprioritize unless Give to Africa adds programming in a conflict-affected country. Revisit only if the portfolio shifts.</t>
-        </is>
-      </c>
-      <c r="P13" s="4" t="inlineStr">
-        <is>
-          <t>Window and closing date confirmed; grant size not confirmed</t>
         </is>
       </c>
       <c r="Q13" s="4" t="inlineStr"/>
@@ -1604,52 +1608,52 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>UNDP / GEF Small Grants Programme (SGP) Ghana</t>
+          <t>Conservation, Food and Health Foundation (CFH)</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Multilateral (UNDP / Global Environment Facility)</t>
+          <t>Private foundation (US)</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>CLOSED - annual, reopens approx. Feb-Mar</t>
+          <t>OPEN - two cycles a year, concept application first</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Up to $30,000 per initiative</t>
+          <t>$25,000 - $50,000 per year; grants awarded for one or two years, year two contingent on progress</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>2026 round closed Mar 13, 2026 (window ran Feb 23 - Mar 13). Expect a similar window in 2027.</t>
+          <t>Two concept-application cycles annually; grants awarded Jul 1 and Dec 1. Next concept deadline reported as mid-December - CONFIRM exact date on the funder's portal.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>2027-03-13</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Local Ghanaian NGOs/non-profits with valid Registrar General's Department and Social Welfare certificates, or CBOs / social enterprises recognized by the District Assembly and Ghana EPA. the Minerals Development Fund (MDF), Ghana would be the applicant; Give to Africa cannot apply directly.</t>
+          <t>Non-profits, NGOs, CSOs, CBOs, universities and academic institutions. Work must be in low- and lower-middle-income countries in Africa, Asia, Latin America or the Middle East - Ghana qualifies. Does NOT fund businesses, government agencies, humanitarian aid organisations, other foundations or churches. Crucially, the requirement is on where the WORK happens, not where the applicant is registered, so Give to Africa appears eligible to apply DIRECTLY as a US 501(c)(3).</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>EXCELLENT strategic fit. The 2026 priority geography was the Black Volta Basin - Wa-West (Upper West), Bole, Sawla-Tuna-Kalba and Central Gonja (Savannah Region) - which is the same northern Ghana shea-gathering belt the the Minerals Development Fund (MDF), Ghana partnership already works in. Focus areas include sustainable agriculture and community-based conservation.</t>
+          <t>STRONGEST DIRECT-APPLY FIT FOUND. Their three focus areas map onto the Ghana programme almost line for line: Conservation (climate change mitigation, local capacity building - shea parklands), Food (sustainable agriculture, small-scale farmer support - shea processing and women's collectives), Health (environmental and occupational health - the PPE procurement for ~1,000 women). They fund pilot projects, new initiatives, training and technical assistance, which is exactly the design-stage facility's profile.</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>https://www.undp.org/ghana</t>
+          <t>https://cfhfoundation.grantsmanagement08.com/</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>not publicly listed (proposal guidelines and template are posted with each call on the UNDP Ghana site)</t>
+          <t>not publicly listed</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
@@ -1657,27 +1661,31 @@
           <t>not publicly listed</t>
         </is>
       </c>
-      <c r="M14" s="7" t="inlineStr">
-        <is>
-          <t>NO OPEN CALL - the 2026 round closed Mar 13. Calls are posted on the UNDP Ghana site and the country page at https://sgp.undp.org (Ghana). CONTACT: the 2026 call published akosua.bireduaa.aninakwa@undp.org for enquiries - email to confirm the 2027 timetable. the Minerals Development Fund (MDF), Ghana must be the applicant and needs valid Registrar General + Social Welfare certificates.</t>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>APPLY HERE: https://cfhfoundation.grantsmanagement08.com/?page_id=6 - online two-phase system. Stage 1 is a SHORT concept application; a limited number are invited to full proposal. Confirm the current cycle's concept deadline on the portal before writing.</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>https://www.undp.org/ghana/press-releases/2026-call-proposals-gef-small-grant-programme-ghana</t>
+          <t>https://cfhfoundation.grantsmanagement08.com/?page_id=6</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>Put a calendar reminder for early February 2027. Confirm now that the Minerals Development Fund (MDF), Ghana's Registrar General and Social Welfare certificates are current - that paperwork is the usual disqualifier, and it takes months to fix.</t>
+          <t>Highest-value new lead. Confirm the next concept deadline on their portal, then submit a concept for the PPE and occupational-health component or the shea parkland conservation angle - both are cleaner fits than the factory build, since CFH funds pilots and technical assistance rather than capital works.</t>
         </is>
       </c>
       <c r="P14" s="4" t="inlineStr">
         <is>
-          <t>Amount, deadline, eligibility and priority districts confirmed across multiple listings</t>
-        </is>
-      </c>
-      <c r="Q14" s="4" t="inlineStr"/>
+          <t>Focus areas, grant size, eligibility categories, two-phase process and award dates confirmed across multiple sources. NEEDS VERIFICATION on the exact next concept deadline - sources give conflicting dates. Confirm on the portal.</t>
+        </is>
+      </c>
+      <c r="Q14" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="96" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
@@ -1687,47 +1695,47 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>WACSI / Wilde Ganzen - Match Funding for Civil Society Organisations in Ghana</t>
+          <t>UN Women's Peace &amp; Humanitarian Fund (WPHF) - Rapid Response Window</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Foundation (regional intermediary)</t>
+          <t>Multilateral (UN)</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>CLOSED - annual, 2026 round closed Apr 27</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Up to $5,000 in match funding, plus coaching and a small kick-start grant</t>
+          <t>Not published in the summary reviewed</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>2026 round closed Apr 27, 2026. Expect a similar spring window in 2027.</t>
+          <t>Concept notes accepted through Dec 31, 2026</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>2027-04-27</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Civil society organisations in Ghana. Organisations must raise at least 50% of project funds LOCALLY - the fund matches up to 50%. Delivered with the Change the Game Academy, which focuses on local fundraising capacity.</t>
+          <t>International and regional NGOs partnering under the Rapid Response Window, in ODA-eligible countries with active peace processes.</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Small money, but unusually well aligned in method. The whole premise - mobilizing local resources and matching them - is what YENDAA does as a platform. A win here is a credible proof point for YENDAA's local-giving thesis, and the coaching component has standalone value for the fiscal sponsorship cohort.</t>
+          <t>WEAK fit. Ghana has no active peace process, so the window's core criterion is not met. Listed only for completeness on the multilateral side.</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>https://wacsi.org</t>
+          <t>https://wphfund.org</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
@@ -1740,24 +1748,24 @@
           <t>not publicly listed</t>
         </is>
       </c>
-      <c r="M15" s="7" t="inlineStr">
-        <is>
-          <t>NO OPEN CALL - the 2026 round closed Apr 27. CALL PAGE: https://wacsi.org/call-for-applications-match-funding-for-civil-society-organisations-in-ghana-2026/ The Terms of Reference and application form download from wacsi.org when a round is live. Ghana-registered CSOs only, and you must raise 50% locally first.</t>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>CALLS ARE POSTED AT: https://wphfund.org - open calls appear there as they launch, each with its own submission instructions. No standing portal. Weak fit for Ghana regardless.</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>https://wacsi.org/call-for-applications-match-funding-for-civil-society-organisations-in-ghana-2026/</t>
+          <t>https://wphfund.org/call-for-proposals-for-rapid-response-window-i-rngo-partners/</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>Calendar for March 2027. Worth approaching WACSI now as a relationship rather than an applicant - they are a regional hub for exactly the West African CSOs YENDAA wants to list.</t>
+          <t>Deprioritize unless Give to Africa adds programming in a conflict-affected country. Revisit only if the portfolio shifts.</t>
         </is>
       </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>Amount, match requirement, partners and deadline confirmed</t>
+          <t>Window and closing date confirmed; grant size not confirmed</t>
         </is>
       </c>
       <c r="Q15" s="4" t="inlineStr"/>
@@ -1770,52 +1778,52 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Canada Fund for Local Initiatives (CFLI) - Ghana</t>
+          <t>UNDP / GEF Small Grants Programme (SGP) Ghana</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Foreign government (Global Affairs Canada)</t>
+          <t>Multilateral (UNDP / Global Environment Facility)</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>CLOSED - annual, reopens approx. Feb-Apr</t>
+          <t>CLOSED - annual, reopens approx. Feb-Mar</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>CAD $25,000 - $45,000 average per project (CAD $200,000 total Ghana envelope)</t>
+          <t>Up to $30,000 per initiative</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>2026 round closed May 10, 2026. Expect the 2027 call around Feb-Apr 2027.</t>
+          <t>2026 round closed Mar 13, 2026 (window ran Feb 23 - Mar 13). Expect a similar window in 2027.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>2027-04-30</t>
+          <t>2027-03-13</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Broad and unusually favorable: local NGOs and non-profits, local academic institutions, AND international non-governmental organizations working on local development activities. Give to Africa appears eligible to apply directly.</t>
+          <t>Local Ghanaian NGOs/non-profits with valid Registrar General's Department and Social Welfare certificates, or CBOs / social enterprises recognized by the District Assembly and Ghana EPA. the Minerals Development Fund (MDF), Ghana would be the applicant; Give to Africa cannot apply directly.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>2026 Ghana themes were democratic governance / human rights and peace &amp; security, with gender equality as a cross-cutting theme. Themes rotate year to year - if a 2027 theme touches women's economic empowerment or climate, the the Minerals Development Fund (MDF), Ghana shea work fits cleanly.</t>
+          <t>EXCELLENT strategic fit. The 2026 priority geography was the Black Volta Basin - Wa-West (Upper West), Bole, Sawla-Tuna-Kalba and Central Gonja (Savannah Region) - which is the same northern Ghana shea-gathering belt the the Minerals Development Fund (MDF), Ghana partnership already works in. Focus areas include sustainable agriculture and community-based conservation.</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>https://www.international.gc.ca/world-monde/funding-financement/cfli-fcil/ghana.aspx?lang=eng</t>
+          <t>https://www.undp.org/ghana</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>ghanacfli@international.gc.ca</t>
+          <t>not publicly listed (proposal guidelines and template are posted with each call on the UNDP Ghana site)</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -1825,22 +1833,22 @@
       </c>
       <c r="M16" s="7" t="inlineStr">
         <is>
-          <t>NO OPEN CALL - 2026 round closed May 10. COUNTRY PAGE: https://www.international.gc.ca/world-monde/funding-financement/cfli-fcil/ghana.aspx?lang=eng When open, apply either through the Collaboration@International (C@I) portal - which needs a Government of Canada GCKey username first - or by emailing the completed application form and budget to ghanacfli@international.gc.ca. A gender-based analysis is mandatory. Email now to be notified for 2027.</t>
+          <t>NO OPEN CALL - the 2026 round closed Mar 13. Calls are posted on the UNDP Ghana site and the country page at https://sgp.undp.org (Ghana). CONTACT: the 2026 call published akosua.bireduaa.aninakwa@undp.org for enquiries - email to confirm the 2027 timetable. the Minerals Development Fund (MDF), Ghana must be the applicant and needs valid Registrar General + Social Welfare certificates.</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>https://www.international.gc.ca/world-monde/funding-financement/cfli-fcil/ghana.aspx?lang=eng</t>
+          <t>https://www.undp.org/ghana/press-releases/2026-call-proposals-gef-small-grant-programme-ghana</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>Email ghanacfli@international.gc.ca now to ask to be notified when the 2027 call opens, and ask what the 2027 thematic priorities will be. This is one of the few government funders on this list where Give to Africa can be the direct applicant.</t>
+          <t>Put a calendar reminder for early February 2027. Confirm now that the Minerals Development Fund (MDF), Ghana's Registrar General and Social Welfare certificates are current - that paperwork is the usual disqualifier, and it takes months to fix.</t>
         </is>
       </c>
       <c r="P16" s="4" t="inlineStr">
         <is>
-          <t>Amounts, deadline, eligibility and contact email confirmed</t>
+          <t>Amount, deadline, eligibility and priority districts confirmed across multiple listings</t>
         </is>
       </c>
       <c r="Q16" s="4" t="inlineStr"/>
@@ -1853,52 +1861,52 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Investing for Employment (IFE) / Invest for Jobs - Ghana Call for Proposals</t>
+          <t>WACSI / Wilde Ganzen - Match Funding for Civil Society Organisations in Ghana</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Foreign government (German development bank KfW)</t>
+          <t>Foundation (regional intermediary)</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>CLOSED - annual, window ran Mar 20 - Jun 1 in 2026</t>
+          <t>CLOSED - annual, 2026 round closed Apr 27</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>EUR 800,000 - EUR 10,000,000 per project. Non-profit projects with no revenue generation are covered up to 90% of investment costs; non-profit with revenue generation up to 75%.</t>
+          <t>Up to $5,000 in match funding, plus coaching and a small kick-start grant</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>2026 window closed Jun 1, 2026 (17:00 CEST). Expect a similar Mar-Jun window in 2027.</t>
+          <t>2026 round closed Apr 27, 2026. Expect a similar spring window in 2027.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>2027-06-01</t>
+          <t>2027-04-27</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Private companies as well as public and NON-PROFIT organisations. All projects must create jobs in the private sector. Two-stage: concept note via the SmartME portal first, full proposal by invitation.</t>
+          <t>Civil society organisations in Ghana. Organisations must raise at least 50% of project funds LOCALLY - the fund matches up to 50%. Delivered with the Change the Game Academy, which focuses on local fundraising capacity.</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>BEST NEW FIND. The the Minerals Development Fund (MDF), Ghana shea butter factories are a job-creation investment in exactly the country and sector IFE funds, and the 90% cost coverage for non-revenue non-profit projects is unusually generous. Scale is far above anything else on this list.</t>
+          <t>Small money, but unusually well aligned in method. The whole premise - mobilizing local resources and matching them - is what YENDAA does as a platform. A win here is a credible proof point for YENDAA's local-giving thesis, and the coaching component has standalone value for the fiscal sponsorship cohort.</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>https://invest-for-jobs.com/en/investing-for-employment</t>
+          <t>https://wacsi.org</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>cfp-ife.2026@invest-for-jobs.com (2026 cycle address - expect the year to change for 2027)</t>
+          <t>not publicly listed</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -1908,22 +1916,22 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>NO OPEN GHANA CALL - the Ghana window closed Jun 1, 2026. A different window (Cote d'Ivoire, Egypt, Morocco) runs Apr 15 - Jun 30, 2026, which shows the cycle is live and rotating. ALL CALLS: https://invest-for-jobs.com/en/calls-for-proposals-overview Applications are submitted ONLY through the SmartME online platform - set up an account and watch the tutorials now: https://invest-for-jobs.com/en/introduction-to-smartme Stage 1 is a concept note scored on jobs created. Email cfp-ife.2026@invest-for-jobs.com to be notified.</t>
+          <t>NO OPEN CALL - the 2026 round closed Apr 27. CALL PAGE: https://wacsi.org/call-for-applications-match-funding-for-civil-society-organisations-in-ghana-2026/ The Terms of Reference and application form download from wacsi.org when a round is live. Ghana-registered CSOs only, and you must raise 50% locally first.</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>https://invest-for-jobs.com/en/call-for-proposals-march-april-2026</t>
+          <t>https://wacsi.org/call-for-applications-match-funding-for-civil-society-organisations-in-ghana-2026/</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>Email the CfP address now to ask to be notified when the 2027 window opens and to confirm whether a U.S. 501(c)(3) can apply directly or must partner with the Minerals Development Fund (MDF), Ghana. Start modelling the factory job-creation numbers - that is the metric IFE selects on.</t>
+          <t>Calendar for March 2027. Worth approaching WACSI now as a relationship rather than an applicant - they are a regional hub for exactly the West African CSOs YENDAA wants to list.</t>
         </is>
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>Amounts, deadline, cost-coverage tiers, eligibility and contact email confirmed across KfW/GTAI/Invest-for-Jobs listings</t>
+          <t>Amount, match requirement, partners and deadline confirmed</t>
         </is>
       </c>
       <c r="Q17" s="4" t="inlineStr"/>
@@ -1936,52 +1944,52 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Common Fund for Commodities (CFC) - Annual Call for Proposals</t>
+          <t>Canada Fund for Local Initiatives (CFLI) - Ghana</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Multilateral (intergovernmental commodity body)</t>
+          <t>Foreign government (Global Affairs Canada)</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>CLOSED - 28th call closed Apr 1, 2026; watch for the 29th</t>
+          <t>CLOSED - annual, reopens approx. Feb-Apr</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Up to $1,500,000 (regular) / $300,000 (fast-track) - note: primarily LOANS and debt instruments, not pure grants</t>
+          <t>CAD $25,000 - $45,000 average per project (CAD $200,000 total Ghana envelope)</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>28th call closed Apr 1, 2026</t>
+          <t>2026 round closed May 10, 2026. Expect the 2027 call around Feb-Apr 2027.</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>2027-04-30</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>SMEs, cooperatives, social enterprises, NGOs and public/private entities based or operating in one of 101 CFC member countries (Ghana is a member). Requires a minimum 3-year operating history and a financially viable project.</t>
+          <t>Broad and unusually favorable: local NGOs and non-profits, local academic institutions, AND international non-governmental organizations working on local development activities. Give to Africa appears eligible to apply directly.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Strong thematic fit for the shea value chain. CFC's stated priorities include local value addition, regenerative agriculture and women's entrepreneurship - the shea butter factory model hits all three. Be aware the instrument is mostly debt, so this suits the revenue-generating factory rather than grant-funded programming.</t>
+          <t>2026 Ghana themes were democratic governance / human rights and peace &amp; security, with gender equality as a cross-cutting theme. Themes rotate year to year - if a 2027 theme touches women's economic empowerment or climate, the the Minerals Development Fund (MDF), Ghana shea work fits cleanly.</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>https://www.common-fund.org</t>
+          <t>https://www.international.gc.ca/world-monde/funding-financement/cfli-fcil/ghana.aspx?lang=eng</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>not publicly listed</t>
+          <t>ghanacfli@international.gc.ca</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -1989,24 +1997,24 @@
           <t>not publicly listed</t>
         </is>
       </c>
-      <c r="M18" s="4" t="inlineStr">
-        <is>
-          <t>CALL PAGE: https://www.common-fund.org/call-for-proposals - the application form is downloadable there when a call is open. The 28th call closed Apr 1, 2026. Two-stage; English only; requires a 3-year operating track record. Mostly loans, not grants.</t>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>NO OPEN CALL - 2026 round closed May 10. COUNTRY PAGE: https://www.international.gc.ca/world-monde/funding-financement/cfli-fcil/ghana.aspx?lang=eng When open, apply either through the Collaboration@International (C@I) portal - which needs a Government of Canada GCKey username first - or by emailing the completed application form and budget to ghanacfli@international.gc.ca. A gender-based analysis is mandatory. Email now to be notified for 2027.</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>https://www.common-fund.org/call-for-proposals</t>
+          <t>https://www.international.gc.ca/world-monde/funding-financement/cfli-fcil/ghana.aspx?lang=eng</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>Watch for the 29th call announcement. Before applying, decide whether the Minerals Development Fund (MDF), Ghana's factory model can service debt - if not, this is the wrong instrument regardless of fit.</t>
+          <t>Email ghanacfli@international.gc.ca now to ask to be notified when the 2027 call opens, and ask what the 2027 thematic priorities will be. This is one of the few government funders on this list where Give to Africa can be the direct applicant.</t>
         </is>
       </c>
       <c r="P18" s="4" t="inlineStr">
         <is>
-          <t>Amounts, deadline, eligibility and instrument type confirmed</t>
+          <t>Amounts, deadline, eligibility and contact email confirmed</t>
         </is>
       </c>
       <c r="Q18" s="4" t="inlineStr"/>
@@ -2019,52 +2027,52 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Dana Foundation - 2026 Grants Programme</t>
+          <t>Investing for Employment (IFE) / Invest for Jobs - Ghana Call for Proposals</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Foreign government (German development bank KfW)</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>NEEDS VERIFICATION - sources give conflicting deadlines</t>
+          <t>CLOSED - annual, window ran Mar 20 - Jun 1 in 2026</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>EUR 50,000 - EUR 150,000 per organization (sources differ)</t>
+          <t>EUR 800,000 - EUR 10,000,000 per project. Non-profit projects with no revenue generation are covered up to 90% of investment costs; non-profit with revenue generation up to 75%.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Conflicting: one source says May 5, 2026 (passed); another says Dec 31, 2026</t>
+          <t>2026 window closed Jun 1, 2026 (17:00 CEST). Expect a similar Mar-Jun window in 2027.</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>2027-06-01</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Locally led and governed organizations in low- or middle-income countries, generally with annual budgets under EUR 500,000, working across multiple dimensions of poverty at once.</t>
+          <t>Private companies as well as public and NON-PROFIT organisations. All projects must create jobs in the private sector. Two-stage: concept note via the SmartME portal first, full proposal by invitation.</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit. 'Locally led and governed' may exclude a U.S.-headquartered 501(c)(3) - but it is a strong fit for the African organizations in the fiscal sponsorship cohort, which is itself a pitchable angle.</t>
+          <t>BEST NEW FIND. The the Minerals Development Fund (MDF), Ghana shea butter factories are a job-creation investment in exactly the country and sector IFE funds, and the 90% cost coverage for non-revenue non-profit projects is unusually generous. Scale is far above anything else on this list.</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>https://invest-for-jobs.com/en/investing-for-employment</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>not publicly listed</t>
+          <t>cfp-ife.2026@invest-for-jobs.com (2026 cycle address - expect the year to change for 2027)</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
@@ -2074,22 +2082,22 @@
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>NO VERIFIED APPLICATION URL FOUND. This entry came from an aggregator roundup and the funder's own grants page could not be confirmed. Do not spend time on it until you verify the funder, the real deadline, and whether a US-based sponsor is eligible.</t>
+          <t>NO OPEN GHANA CALL - the Ghana window closed Jun 1, 2026. A different window (Cote d'Ivoire, Egypt, Morocco) runs Apr 15 - Jun 30, 2026, which shows the cycle is live and rotating. ALL CALLS: https://invest-for-jobs.com/en/calls-for-proposals-overview Applications are submitted ONLY through the SmartME online platform - set up an account and watch the tutorials now: https://invest-for-jobs.com/en/introduction-to-smartme Stage 1 is a concept note scored on jobs created. Email cfp-ife.2026@invest-for-jobs.com to be notified.</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>https://africanngos.org/2026/06/09/african-ngo-funding-opportunities-june-july-2026/</t>
+          <t>https://invest-for-jobs.com/en/call-for-proposals-march-april-2026</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>Verify the real deadline and whether a U.S.-based sponsor is eligible before investing effort. If only locally led orgs qualify, redirect this to fiscal sponsorship cohort members.</t>
-        </is>
-      </c>
-      <c r="P19" s="8" t="inlineStr">
-        <is>
-          <t>NEEDS VERIFICATION - deadline and grant size both inconsistent across sources; funder's own site not confirmed</t>
+          <t>Email the CfP address now to ask to be notified when the 2027 window opens and to confirm whether a U.S. 501(c)(3) can apply directly or must partner with the Minerals Development Fund (MDF), Ghana. Start modelling the factory job-creation numbers - that is the metric IFE selects on.</t>
+        </is>
+      </c>
+      <c r="P19" s="4" t="inlineStr">
+        <is>
+          <t>Amounts, deadline, cost-coverage tiers, eligibility and contact email confirmed across KfW/GTAI/Invest-for-Jobs listings</t>
         </is>
       </c>
       <c r="Q19" s="4" t="inlineStr"/>
@@ -2102,27 +2110,27 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>U.S. African Development Foundation (USADF)</t>
+          <t>Common Fund for Commodities (CFC) - Annual Call for Proposals</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>U.S. Government (independent federal agency)</t>
+          <t>Multilateral (intergovernmental commodity body)</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>NOT ACCEPTING APPLICATIONS - per USADF's own apply page</t>
+          <t>CLOSED - 28th call closed Apr 1, 2026; watch for the 29th</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Up to $250,000</t>
+          <t>Up to $1,500,000 (regular) / $300,000 (fast-track) - note: primarily LOANS and debt instruments, not pure grants</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Varies by country call - check usadf.gov for the current Ghana call</t>
+          <t>28th call closed Apr 1, 2026</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -2132,22 +2140,22 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Applicant must be a 100% African-owned enterprise, cooperative, producer group or processor in an eligible country. Give to Africa is NOT directly eligible - the shea cooperative or the Minerals Development Fund (MDF), Ghana would be the grantee, with Give to Africa providing proposal and compliance support.</t>
+          <t>SMEs, cooperatives, social enterprises, NGOs and public/private entities based or operating in one of 101 CFC member countries (Ghana is a member). Requires a minimum 3-year operating history and a financially viable project.</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Strong on-mission fit - USADF funds exactly this kind of agricultural processor and women's producer group - but there is nothing to apply to at present.</t>
+          <t>Strong thematic fit for the shea value chain. CFC's stated priorities include local value addition, regenerative agriculture and women's entrepreneurship - the shea butter factory model hits all three. Be aware the instrument is mostly debt, so this suits the revenue-generating factory rather than grant-funded programming.</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>https://usadf.gov</t>
+          <t>https://www.common-fund.org</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>not publicly listed (each country call names its own submission address)</t>
+          <t>not publicly listed</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
@@ -2155,24 +2163,24 @@
           <t>not publicly listed</t>
         </is>
       </c>
-      <c r="M20" s="6" t="inlineStr">
-        <is>
-          <t>APPLY PAGE: https://www.usadf.gov/apply - but that page currently states applications are NOT being accepted. There is no open Ghana call to apply to right now. Check the page periodically; when a country call opens it names its own submission email address.</t>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>CALL PAGE: https://www.common-fund.org/call-for-proposals - the application form is downloadable there when a call is open. The 28th call closed Apr 1, 2026. Two-stage; English only; requires a 3-year operating track record. Mostly loans, not grants.</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>https://usadf.gov/resources</t>
+          <t>https://www.common-fund.org/call-for-proposals</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>Confirm whether Ghana is in the current eligible-country list, then position the shea cooperative as applicant. Even at partner-support level this is the largest realistic U.S. government award on this list.</t>
-        </is>
-      </c>
-      <c r="P20" s="8" t="inlineStr">
-        <is>
-          <t>CORRECTED Jul 29, 2026. Previously listed as open with periodic country calls. USADF's own apply page states applications are not being accepted at this time. Ghana eligibility also remains unconfirmed - sources conflict.</t>
+          <t>Watch for the 29th call announcement. Before applying, decide whether the Minerals Development Fund (MDF), Ghana's factory model can service debt - if not, this is the wrong instrument regardless of fit.</t>
+        </is>
+      </c>
+      <c r="P20" s="4" t="inlineStr">
+        <is>
+          <t>Amounts, deadline, eligibility and instrument type confirmed</t>
         </is>
       </c>
       <c r="Q20" s="4" t="inlineStr"/>
@@ -2185,243 +2193,243 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
+          <t>Dana Foundation - 2026 Grants Programme</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION - sources give conflicting deadlines</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>EUR 50,000 - EUR 150,000 per organization (sources differ)</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Conflicting: one source says May 5, 2026 (passed); another says Dec 31, 2026</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Locally led and governed organizations in low- or middle-income countries, generally with annual budgets under EUR 500,000, working across multiple dimensions of poverty at once.</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Moderate fit. 'Locally led and governed' may exclude a U.S.-headquartered 501(c)(3) - but it is a strong fit for the African organizations in the fiscal sponsorship cohort, which is itself a pitchable angle.</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>NO VERIFIED APPLICATION URL FOUND. This entry came from an aggregator roundup and the funder's own grants page could not be confirmed. Do not spend time on it until you verify the funder, the real deadline, and whether a US-based sponsor is eligible.</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>https://africanngos.org/2026/06/09/african-ngo-funding-opportunities-june-july-2026/</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>Verify the real deadline and whether a U.S.-based sponsor is eligible before investing effort. If only locally led orgs qualify, redirect this to fiscal sponsorship cohort members.</t>
+        </is>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION - deadline and grant size both inconsistent across sources; funder's own site not confirmed</t>
+        </is>
+      </c>
+      <c r="Q21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22" ht="96" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>3 - Calendar for next cycle</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>U.S. African Development Foundation (USADF)</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>U.S. Government (independent federal agency)</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>NOT ACCEPTING APPLICATIONS - per USADF's own apply page</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Up to $250,000</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Varies by country call - check usadf.gov for the current Ghana call</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Applicant must be a 100% African-owned enterprise, cooperative, producer group or processor in an eligible country. Give to Africa is NOT directly eligible - the shea cooperative or the Minerals Development Fund (MDF), Ghana would be the grantee, with Give to Africa providing proposal and compliance support.</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Strong on-mission fit - USADF funds exactly this kind of agricultural processor and women's producer group - but there is nothing to apply to at present.</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>https://usadf.gov</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed (each country call names its own submission address)</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M22" s="6" t="inlineStr">
+        <is>
+          <t>APPLY PAGE: https://www.usadf.gov/apply - but that page currently states applications are NOT being accepted. There is no open Ghana call to apply to right now. Check the page periodically; when a country call opens it names its own submission email address.</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>https://usadf.gov/resources</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>Confirm whether Ghana is in the current eligible-country list, then position the shea cooperative as applicant. Even at partner-support level this is the largest realistic U.S. government award on this list.</t>
+        </is>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>CORRECTED Jul 29, 2026. Previously listed as open with periodic country calls. USADF's own apply page states applications are not being accepted at this time. Ghana eligibility also remains unconfirmed - sources conflict.</t>
+        </is>
+      </c>
+      <c r="Q22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23" ht="96" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>3 - Calendar for next cycle</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
           <t>United Nations Democracy Fund (UNDEF)</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Multilateral (UN)</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>CLOSED - annual window, 2026 round not yet announced</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Up to $300,000 per project (two-year projects)</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Annual window, historically about a month long (a recent round ran Nov 1-30)</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>Civil society organizations and NGOs promoting democracy; preference for countries in democratic transition and consolidation, least developed countries, and low/middle-income countries.</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>Moderate fit. Would need to be framed around civil-society strengthening - the fiscal sponsorship program and YENDAA's transparency/verification infrastructure for African-led organizations is the most credible angle.</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr">
         <is>
           <t>https://www.un.org/democracyfund/en</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M21" s="6" t="inlineStr">
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M23" s="6" t="inlineStr">
         <is>
           <t>APPLY VIA THE OPPS PORTAL: https://www.un.org/democracyfund/en/content/how-apply-online-project-proposal-system-opps You must REGISTER YOUR ORGANIZATION FIRST to receive a login - do that before the window opens, since the window is short (historically about a month, often November). Technical support: undefproposal@un.org. Draft offline using their blank proposal form, then paste in.</t>
         </is>
       </c>
-      <c r="N21" s="4" t="inlineStr">
+      <c r="N23" s="4" t="inlineStr">
         <is>
           <t>https://www.un.org/democracyfund/en/apply-for-funding</t>
         </is>
       </c>
-      <c r="O21" s="4" t="inlineStr">
+      <c r="O23" s="4" t="inlineStr">
         <is>
           <t>Check the UNDEF site monthly from October onward. The window is short and there is no extension, so a draft concept must exist before it opens.</t>
         </is>
       </c>
-      <c r="P21" s="4" t="inlineStr">
+      <c r="P23" s="4" t="inlineStr">
         <is>
           <t>Grant ceiling and eligibility confirmed; 2026 round dates not yet published</t>
-        </is>
-      </c>
-      <c r="Q21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22" ht="96" customHeight="1">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t>4 - Low priority</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>USDA Foreign Agricultural Service - McGovern-Dole International Food for Education FY2026</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>U.S. Government (federal)</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>CLOSED for FY2026</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Not published in the summary reviewed (multi-million, multi-year)</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Closed Jun 22, 2026</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>Non-profits, cooperatives, universities and similar entities. Non-priority countries are accepted but rarely funded.</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>Poor fit. FY2026 priority countries in West Africa were Guinea (Conakry) and Liberia - not Ghana. Education focus is school feeding and child nutrition, not workforce development.</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>https://www.fas.usda.gov</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M22" s="7" t="inlineStr">
-        <is>
-          <t>CLOSED for FY2026. Future rounds post on grants.gov and at fas.usda.gov. Ghana is not a priority country - watch the FY2027 priority-country announcement before investing any time.</t>
-        </is>
-      </c>
-      <c r="N22" s="4" t="inlineStr">
-        <is>
-          <t>https://www.fas.usda.gov/newsroom/stakeholder-notice-usda-publishes-fy-2026-notice-funding-opportunity-mcgovern-dole-program</t>
-        </is>
-      </c>
-      <c r="O22" s="4" t="inlineStr">
-        <is>
-          <t>Skip. Listed so the FY2027 priority-country announcement can be checked - if Ghana is added, reassess.</t>
-        </is>
-      </c>
-      <c r="P22" s="4" t="inlineStr">
-        <is>
-          <t>Deadline and priority countries confirmed</t>
-        </is>
-      </c>
-      <c r="Q22" s="4" t="inlineStr"/>
-    </row>
-    <row r="23" ht="96" customHeight="1">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>4 - Low priority</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>USDA Foreign Agricultural Service - Food for Progress FY2026</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>U.S. Government (federal)</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
-        <is>
-          <t>CLOSED for FY2026</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>$28,000,000 - $35,000,000 per award (up to $226M total)</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Closed Jul 6, 2026</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>Governments, intergovernmental organizations, PVOs, non-profit agricultural organizations and cooperatives, NGOs, universities, and other private entities. Award sizes require major institutional capacity.</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t>Poor fit at current scale. FY2026 priority countries were Bangladesh, Bolivia, Ecuador, Morocco, the Philippines, Sri Lanka and Thailand - Ghana was not among them.</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>https://www.fas.usda.gov/programs/food-progress</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M23" s="7" t="inlineStr">
-        <is>
-          <t>CLOSED for FY2026. Future rounds post on grants.gov and at https://www.fas.usda.gov/programs/food-progress - not viable at your current scale regardless.</t>
-        </is>
-      </c>
-      <c r="N23" s="4" t="inlineStr">
-        <is>
-          <t>https://www.fas.usda.gov/newsroom/usda-publishes-fy-2026-notices-funding-opportunity-food-progress</t>
-        </is>
-      </c>
-      <c r="O23" s="4" t="inlineStr">
-        <is>
-          <t>Not viable now - award sizes are far above Give to Africa's current capacity and Ghana is off the priority list. Revisit only as a sub-awardee to a large prime.</t>
-        </is>
-      </c>
-      <c r="P23" s="4" t="inlineStr">
-        <is>
-          <t>Amounts, deadline and priority countries confirmed</t>
         </is>
       </c>
       <c r="Q23" s="4" t="inlineStr"/>
@@ -2434,47 +2442,47 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>UN Women - Spotlight Initiative Africa Regional Programme (SIARP) 2.0</t>
+          <t>USDA Foreign Agricultural Service - McGovern-Dole International Food for Education FY2026</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Multilateral (UN)</t>
+          <t>U.S. Government (federal)</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>CLOSED - deadline passed Jul 27, 2026</t>
+          <t>CLOSED for FY2026</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>$110,000 - $548,000 (27-month projects, Oct 2026 - Dec 2028)</t>
+          <t>Not published in the summary reviewed (multi-million, multi-year)</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Jul 27, 2026, 5pm East Africa Time</t>
+          <t>Closed Jun 22, 2026</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>CSOs, women's rights organizations, coalitions and networks operating at continental, regional, sub-regional or multi-country level in Africa, with demonstrated gender-equality programming experience.</t>
+          <t>Non-profits, cooperatives, universities and similar entities. Non-priority countries are accepted but rarely funded.</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Would have been a good multi-country fit given the cross-border structure, but the thematic focus (ending violence against women and girls, SRHR, survivor services) sits outside Give to Africa's four programs.</t>
+          <t>Poor fit. FY2026 priority countries in West Africa were Guinea (Conakry) and Liberia - not Ghana. Education focus is school feeding and child nutrition, not workforce development.</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>https://africa.unwomen.org</t>
+          <t>https://www.fas.usda.gov</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
@@ -2489,22 +2497,22 @@
       </c>
       <c r="M24" s="7" t="inlineStr">
         <is>
-          <t>CLOSED - deadline passed Jul 27, 2026. Future UN Women Africa calls are posted at https://africa.unwomen.org under programme implementation.</t>
+          <t>CLOSED for FY2026. Future rounds post on grants.gov and at fas.usda.gov. Ghana is not a priority country - watch the FY2027 priority-country announcement before investing any time.</t>
         </is>
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>https://africa.unwomen.org/en/programme-implementation/2026/06/call-for-proposals-for-civil-society-partnerships-for-implementation-of-the-spotlight-initiative-africa-regional-programme-siarp-20</t>
+          <t>https://www.fas.usda.gov/newsroom/stakeholder-notice-usda-publishes-fy-2026-notice-funding-opportunity-mcgovern-dole-program</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>Missed for this cycle. Worth tracking UN Women Africa's calls generally - the multi-country eligibility structure suits Give to Africa's cross-border model better than most funders'.</t>
+          <t>Skip. Listed so the FY2027 priority-country announcement can be checked - if Ghana is added, reassess.</t>
         </is>
       </c>
       <c r="P24" s="4" t="inlineStr">
         <is>
-          <t>Amounts, deadline and eligibility confirmed</t>
+          <t>Deadline and priority countries confirmed</t>
         </is>
       </c>
       <c r="Q24" s="4" t="inlineStr"/>
@@ -2517,83 +2525,336 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
+          <t>USDA Foreign Agricultural Service - Food for Progress FY2026</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>U.S. Government (federal)</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>CLOSED for FY2026</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>$28,000,000 - $35,000,000 per award (up to $226M total)</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Closed Jul 6, 2026</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Governments, intergovernmental organizations, PVOs, non-profit agricultural organizations and cooperatives, NGOs, universities, and other private entities. Award sizes require major institutional capacity.</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Poor fit at current scale. FY2026 priority countries were Bangladesh, Bolivia, Ecuador, Morocco, the Philippines, Sri Lanka and Thailand - Ghana was not among them.</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.fas.usda.gov/programs/food-progress</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="inlineStr">
+        <is>
+          <t>CLOSED for FY2026. Future rounds post on grants.gov and at https://www.fas.usda.gov/programs/food-progress - not viable at your current scale regardless.</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.fas.usda.gov/newsroom/usda-publishes-fy-2026-notices-funding-opportunity-food-progress</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>Not viable now - award sizes are far above Give to Africa's current capacity and Ghana is off the priority list. Revisit only as a sub-awardee to a large prime.</t>
+        </is>
+      </c>
+      <c r="P25" s="4" t="inlineStr">
+        <is>
+          <t>Amounts, deadline and priority countries confirmed</t>
+        </is>
+      </c>
+      <c r="Q25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26" ht="96" customHeight="1">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>4 - Low priority</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>UN Women - Spotlight Initiative Africa Regional Programme (SIARP) 2.0</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Multilateral (UN)</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>CLOSED - deadline passed Jul 27, 2026</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>$110,000 - $548,000 (27-month projects, Oct 2026 - Dec 2028)</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Jul 27, 2026, 5pm East Africa Time</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>CSOs, women's rights organizations, coalitions and networks operating at continental, regional, sub-regional or multi-country level in Africa, with demonstrated gender-equality programming experience.</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>Would have been a good multi-country fit given the cross-border structure, but the thematic focus (ending violence against women and girls, SRHR, survivor services) sits outside Give to Africa's four programs.</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>https://africa.unwomen.org</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M26" s="7" t="inlineStr">
+        <is>
+          <t>CLOSED - deadline passed Jul 27, 2026. Future UN Women Africa calls are posted at https://africa.unwomen.org under programme implementation.</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>https://africa.unwomen.org/en/programme-implementation/2026/06/call-for-proposals-for-civil-society-partnerships-for-implementation-of-the-spotlight-initiative-africa-regional-programme-siarp-20</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>Missed for this cycle. Worth tracking UN Women Africa's calls generally - the multi-country eligibility structure suits Give to Africa's cross-border model better than most funders'.</t>
+        </is>
+      </c>
+      <c r="P26" s="4" t="inlineStr">
+        <is>
+          <t>Amounts, deadline and eligibility confirmed</t>
+        </is>
+      </c>
+      <c r="Q26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27" ht="96" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>4 - Low priority</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Smart &amp; Final Charitable Foundation</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Corporate foundation (US retail)</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>NOT ELIGIBLE - geographic mismatch</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Not published; product and monetary donations</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Reported application deadline Jan 6, 2026 - passed</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>2027-01-06</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Supports nonprofits improving quality of life in communities the COMPANY SERVES - Arizona, California and Nevada. Focus areas: health and wellness, education, hunger relief, team sports and youth development, disaster relief. 501(c)(3) required.</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>NOT A FIT as things stand. Give to Africa is San Diego-registered, but the funded WORK must benefit AZ/CA/NV communities and all four Give to Africa programs operate in Africa. This would only become viable if Give to Africa ran a San Diego-facing program - diaspora engagement, local youth education, volunteer programming.</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.smartandfinal.com</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>323-869-7506 (published foundation contact)</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>NOT ELIGIBLE for current programming - do not apply. Their giving is restricted to communities the company serves in Arizona, California and Nevada.</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.theshareway.com/grant/smart--08852-smart-final-charitable-foundation-donations</t>
+        </is>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t>Do not apply for Africa programming. Recorded so this ground is not re-searched. Revisit only if Give to Africa launches a San Diego-based program - see the note on local corporate funders in the method sheet.</t>
+        </is>
+      </c>
+      <c r="P27" s="4" t="inlineStr">
+        <is>
+          <t>Geographic restriction, focus areas and phone number confirmed. Deadline reported as Jan 6, 2026 and presumed annual.</t>
+        </is>
+      </c>
+      <c r="Q27" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="96" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>4 - Low priority</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
           <t>Segal Family Foundation</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>NOT OPEN - invitation only</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>$10,000 - $100,000+ (averaging approx. $50,000; approx. $15M granted annually)</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>No deadline - does not accept unsolicited applications</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>Grassroots African-led organizations in education, youth empowerment and social entrepreneurship. Grantees come through referral only.</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>Very strong mission fit (trust-based philanthropy for African-led organizations) but there is no application route. This is a relationship-building target, not a proposal target.</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>https://www.segalfamilyfoundation.org</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M25" s="7" t="inlineStr">
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M28" s="7" t="inlineStr">
         <is>
           <t>NO APPLICATION ROUTE - Segal does not accept unsolicited applications and works purely by referral. Do not submit anything. Map who in your network can make a warm introduction.</t>
         </is>
       </c>
-      <c r="N25" s="4" t="inlineStr">
+      <c r="N28" s="4" t="inlineStr">
         <is>
           <t>https://www.segalfamilyfoundation.org/what-we-do/invest/grantmaking/</t>
         </is>
       </c>
-      <c r="O25" s="4" t="inlineStr">
+      <c r="O28" s="4" t="inlineStr">
         <is>
           <t>Do not submit a proposal - it will not be read. Instead, map who in Give to Africa's network already holds a Segal relationship and pursue a warm referral. Their African-led portfolio overlaps heavily with YENDAA's target causes.</t>
         </is>
       </c>
-      <c r="P25" s="4" t="inlineStr">
+      <c r="P28" s="4" t="inlineStr">
         <is>
           <t>Referral-only model and grant range confirmed</t>
         </is>
       </c>
-      <c r="Q25" s="4" t="inlineStr"/>
+      <c r="Q28" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:Q25"/>
+  <autoFilter ref="A2:Q28"/>
   <mergeCells count="1">
     <mergeCell ref="A1:Q1"/>
   </mergeCells>
@@ -2754,7 +3015,7 @@
         </is>
       </c>
       <c r="B20" s="22" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21">
@@ -2774,7 +3035,7 @@
         </is>
       </c>
       <c r="B22" s="23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
@@ -2784,7 +3045,7 @@
         </is>
       </c>
       <c r="B23" s="23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24">
@@ -2794,7 +3055,7 @@
         </is>
       </c>
       <c r="B24" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">

</xml_diff>

<commit_message>
Correct Smart & Final to confirmed prior funder; add California corporate category
Smart & Final was recorded as NOT ELIGIBLE based on a reading of their published
AZ/CA/NV geographic language. Victoria confirms they funded Give to Africa in
2025. An actual award overrides an inference from guidelines - corrected to a
prior funder with an annual renewal action.

Opens the California corporate category on the strength of that precedent: Vons
Foundation (quarterly, employee sponsor via store manager), Sempra (year-round
partnership track, climate framing), and SDG&E (recorded with its explicit
service-area limit and its regranting and capital-project exclusions, which make
it weaker than it first appears).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PULTYHtQSMT98yhFaxzQDo
</commit_message>
<xml_diff>
--- a/Give-to-Africa-Grant-Pipeline-2026.xlsx
+++ b/Give-to-Africa-Grant-Pipeline-2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How to Use + Method" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Grant Pipeline'!$A$2:$Q$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Grant Pipeline'!$A$2:$Q$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q28"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -592,7 +592,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Give to Africa - Grant Pipeline (Government, Multilateral &amp; Foundation)  |  Last updated July 30, 2026  |  26 opportunities tracked</t>
+          <t>Give to Africa - Grant Pipeline (Government, Multilateral &amp; Foundation)  |  Last updated July 30, 2026  |  29 opportunities tracked</t>
         </is>
       </c>
     </row>
@@ -1276,27 +1276,27 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>U.S. Embassy Ghana - Ambassador's Special Self-Help (ASSH) Program</t>
+          <t>San Diego Gas &amp; Electric (SDG&amp;E) - community giving</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>U.S. Government (embassy small grants)</t>
+          <t>Corporate giving (San Diego utility)</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>OPEN - annual cycle, confirm current window</t>
+          <t>OPEN - online application system, cycle dates not confirmed</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>$1,000 - $12,000 (awards typically $2,000 - $10,000)</t>
+          <t>Varies. A one-off $10M Community Assistance Fund made grants of $250,000-$1,000,000, but that was an exceptional initiative, not the standard programme.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Annual cycle - current 2026 window not published online; email the coordinator to confirm</t>
+          <t>Not confirmed for 2026 - check the funding guidelines page</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1306,22 +1306,22 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Applicant must be a non-profit, NGO or CBO registered with the Government of Ghana, or a community association formed at least a year before applying. Give to Africa cannot apply directly - the Minerals Development Fund (MDF), Ghana or a shea cooperative must be the applicant. Requires substantial community contribution (labor, materials, land, expertise).</t>
+          <t>501(c)(3) public charities OPERATING IN AND SERVING San Diego County or select South Orange County ZIP codes. Priorities: environmental programmes, emergency preparedness, public safety, STEM leadership, economic prosperity and workforce development. Explicitly WILL NOT FUND regranting programmes, research, capital projects, endowments, or debt payments.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Climate Resilience / the Minerals Development Fund (MDF), Ghana. A 12-month, community-led shea processing or PPE project is precisely the profile ASSH funds, and the required community contribution is already covered by the existing 80/20 split and 4-to-1 government match.</t>
+          <t>WEAKER THAN IT LOOKS. The service-area requirement is explicit - the funded work must serve San Diego County. Their exclusions also rule out regranting (fiscal sponsorship) and capital projects (the factory). Viable only against a San Diego-based programme, most plausibly workforce development or STEM, which are named priorities.</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>https://gh.usembassy.gov/ambassadors-special-self-help-program/</t>
+          <t>https://www.sdge.com/more-information/community/funding-guidelines</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>AccraSelfHelp@state.gov</t>
+          <t>not publicly listed</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -1331,25 +1331,29 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>PROGRAM PAGE: https://gh.usembassy.gov/education-culture/ambassadors-special-self-help-program/ No live application form is posted between cycles. EMAIL AccraSelfHelp@state.gov to ask for the current Notice of Funding Opportunity and application form. the Minerals Development Fund (MDF), Ghana must be the applicant.</t>
+          <t>GUIDELINES: https://www.sdge.com/more-information/community/funding-guidelines - online grant application system; first-time applicants create a login. Read the exclusions before starting: regranting, research and capital projects are all ineligible.</t>
         </is>
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>https://gh.usembassy.gov/ambassadors-special-self-help-program/</t>
+          <t>https://www.sdge.com/more-information/community/funding-guidelines</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>Email AccraSelfHelp@state.gov this week asking when the next window opens, and have the Minerals Development Fund (MDF), Ghana ready as the named applicant. Small award, but a U.S. Embassy grant is a credential worth more than $12,000 in later proposals.</t>
+          <t>Do not apply for Africa programming - the service-area language here is far more explicit than Smart &amp; Final's. Revisit if a San Diego-facing workforce development or STEM programme is launched.</t>
         </is>
       </c>
       <c r="P10" s="4" t="inlineStr">
         <is>
-          <t>Amounts and eligibility confirmed; current-cycle deadline NOT confirmed - the embassy page has not published a 2026 date</t>
-        </is>
-      </c>
-      <c r="Q10" s="4" t="inlineStr"/>
+          <t>Service area, priorities and exclusions confirmed. Current cycle dates NOT confirmed.</t>
+        </is>
+      </c>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="96" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
@@ -1359,52 +1363,52 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>U.S. Embassy Ghana - Public Diplomacy Section Annual Program Statement (APS)</t>
+          <t>Sempra - Community Partnerships (year-round) and SoCal Climate Champions</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>U.S. Government (embassy small grants)</t>
+          <t>Corporate foundation (San Diego energy)</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>WATCH - last confirmed cycle closed, reissued annually</t>
+          <t>PARTIALLY OPEN - annual community grants closed; partnerships accepted year-round</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>$15,000 - $100,000 (range from the most recently confirmed cycle)</t>
+          <t>Partnerships from $10,000 with no stated ceiling; annual community grants up to $10,000; SoCal Climate Champions reported up to $50,000</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Not currently posted - APS is normally reissued each fiscal year</t>
+          <t>Partnerships: proposals accepted year-round. 2026 community grant cycle closed (Feb 23). Climate Champions cycle not confirmed.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rolling</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Registered non-profits, NGOs, academic institutions and civil society organizations. Two-step: Statement of Interest first, full proposal by invitation. U.S.-based organizations have been eligible in prior Ghana cycles.</t>
+          <t>Nonprofits, with Sempra's giving focused on environmental stewardship, energy education, community resilience and climate solutions. San Diego headquartered company. Confirm geographic requirements before applying.</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Education &amp; Workforce Development - the Bradford University African Philanthropy Studies curriculum is a natural APS project (educational exchange, capacity building, U.S.-Ghana institutional linkage).</t>
+          <t>The climate framing is the opening. Sempra funds environmental stewardship and climate solutions, and Give to Africa's Climate Resilience programme - solar-powered processing and community water - speaks that language. The year-round partnership track avoids waiting for the February cycle.</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>https://gh.usembassy.gov/education-culture/public-affairs-small-grants/</t>
+          <t>https://www.sempra.com/performance/community-giving</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>PASAccraGrant@state.gov</t>
+          <t>not publicly listed</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
@@ -1414,25 +1418,29 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>PROGRAM PAGE: https://gh.usembassy.gov/education-culture/public-affairs-small-grants/ No open call posted. EMAIL PASAccraGrant@state.gov to ask when the next Annual Program Statement is issued. When live, step 1 is a short Statement of Interest, not a full proposal.</t>
+          <t>GUIDELINES: https://www.sempra.com/corporate-giving-guidelines-faq - the annual community grant cycle closed in February, but PARTNERSHIP proposals starting at $10,000 are accepted year-round. That is the route to use now.</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>https://gh.usembassy.gov/education-culture/public-affairs-small-grants/public-diplomacy-section-annual-program-statement-request-for-statements-of-interest/</t>
+          <t>https://www.sempra.com/performance/community-giving</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>Email PASAccraGrant@state.gov to ask when the FY2027 APS will be issued and to be added to any notification list. Draft the Bradford curriculum Statement of Interest now so it is ready the day the APS posts.</t>
+          <t>Pursue the year-round partnership track rather than waiting for February. Lead with solar and climate resilience. Verify whether they require the funded work to be in their service territory - if so, this becomes a San Diego-programme conversation.</t>
         </is>
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>Email address and prior-cycle funding range confirmed; no open 2026 call found</t>
-        </is>
-      </c>
-      <c r="Q11" s="4" t="inlineStr"/>
+          <t>Community grant amounts, February deadline, year-round partnership track and Climate Champions programme confirmed. NEEDS VERIFICATION on whether funded work must be in-territory.</t>
+        </is>
+      </c>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="96" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
@@ -1442,52 +1450,52 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>UK FCDO - Funder Finder / Ghana country office</t>
+          <t>U.S. Embassy Ghana - Ambassador's Special Self-Help (ASSH) Program</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Foreign government (UK)</t>
+          <t>U.S. Government (embassy small grants)</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>MONITORING SOURCE - no Ghana-specific open call identified</t>
+          <t>OPEN - annual cycle, confirm current window</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Varies by programme</t>
+          <t>$1,000 - $12,000 (awards typically $2,000 - $10,000)</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Varies - Funder Finder is a searchable live database</t>
+          <t>Annual cycle - current 2026 window not published online; email the coordinator to confirm</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>rolling</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Varies by call. FCDO funds CSOs through mechanisms such as Aid Connect, which invites proposals from CSO consortia. Bond advises contacting FCDO country offices directly, as some funding is distributed at country level.</t>
+          <t>Applicant must be a non-profit, NGO or CBO registered with the Government of Ghana, or a community association formed at least a year before applying. Give to Africa cannot apply directly - the Minerals Development Fund (MDF), Ghana or a shea cooperative must be the applicant. Requires substantial community contribution (labor, materials, land, expertise).</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>No open call matched to Give to Africa's programs at the time of this search. Listed as a channel to monitor rather than an opportunity - the Ghana Governance Programme shows FCDO does fund Ghanaian civil society.</t>
+          <t>Climate Resilience / the Minerals Development Fund (MDF), Ghana. A 12-month, community-led shea processing or PPE project is precisely the profile ASSH funds, and the required community contribution is already covered by the existing 80/20 split and 4-to-1 government match.</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>https://devtracker.fcdo.gov.uk/countries/GH/projects/</t>
+          <t>https://gh.usembassy.gov/ambassadors-special-self-help-program/</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>not publicly listed</t>
+          <t>AccraSelfHelp@state.gov</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
@@ -1495,24 +1503,24 @@
           <t>not publicly listed</t>
         </is>
       </c>
-      <c r="M12" s="7" t="inlineStr">
-        <is>
-          <t>NO SPECIFIC CALL. Search the FCDO Funder Finder and the UK government funding portal for live opportunities, and see Bond's funding page: https://www.bond.org.uk/resources-support/funding/ Bond specifically advises contacting the FCDO Ghana country office directly, since some funds are distributed at country level.</t>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>PROGRAM PAGE: https://gh.usembassy.gov/education-culture/ambassadors-special-self-help-program/ No live application form is posted between cycles. EMAIL AccraSelfHelp@state.gov to ask for the current Notice of Funding Opportunity and application form. the Minerals Development Fund (MDF), Ghana must be the applicant.</t>
         </is>
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>https://www.bond.org.uk/resources-support/funding/</t>
+          <t>https://gh.usembassy.gov/ambassadors-special-self-help-program/</t>
         </is>
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>Add FCDO Funder Finder to the daily monitor's source rotation. Consider contacting the FCDO Ghana country office directly, which Bond specifically recommends for country-level funds.</t>
+          <t>Email AccraSelfHelp@state.gov this week asking when the next window opens, and have the Minerals Development Fund (MDF), Ghana ready as the named applicant. Small award, but a U.S. Embassy grant is a credential worth more than $12,000 in later proposals.</t>
         </is>
       </c>
       <c r="P12" s="4" t="inlineStr">
         <is>
-          <t>Mechanism and guidance confirmed; NO specific open opportunity found</t>
+          <t>Amounts and eligibility confirmed; current-cycle deadline NOT confirmed - the embassy page has not published a 2026 date</t>
         </is>
       </c>
       <c r="Q12" s="4" t="inlineStr"/>
@@ -1525,333 +1533,333 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t>U.S. Embassy Ghana - Public Diplomacy Section Annual Program Statement (APS)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>U.S. Government (embassy small grants)</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>WATCH - last confirmed cycle closed, reissued annually</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>$15,000 - $100,000 (range from the most recently confirmed cycle)</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Not currently posted - APS is normally reissued each fiscal year</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Registered non-profits, NGOs, academic institutions and civil society organizations. Two-step: Statement of Interest first, full proposal by invitation. U.S.-based organizations have been eligible in prior Ghana cycles.</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Education &amp; Workforce Development - the Bradford University African Philanthropy Studies curriculum is a natural APS project (educational exchange, capacity building, U.S.-Ghana institutional linkage).</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>https://gh.usembassy.gov/education-culture/public-affairs-small-grants/</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>PASAccraGrant@state.gov</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>PROGRAM PAGE: https://gh.usembassy.gov/education-culture/public-affairs-small-grants/ No open call posted. EMAIL PASAccraGrant@state.gov to ask when the next Annual Program Statement is issued. When live, step 1 is a short Statement of Interest, not a full proposal.</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>https://gh.usembassy.gov/education-culture/public-affairs-small-grants/public-diplomacy-section-annual-program-statement-request-for-statements-of-interest/</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>Email PASAccraGrant@state.gov to ask when the FY2027 APS will be issued and to be added to any notification list. Draft the Bradford curriculum Statement of Interest now so it is ready the day the APS posts.</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>Email address and prior-cycle funding range confirmed; no open 2026 call found</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14" ht="96" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>2 - Open / rolling</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>UK FCDO - Funder Finder / Ghana country office</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Foreign government (UK)</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>MONITORING SOURCE - no Ghana-specific open call identified</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Varies by programme</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Varies - Funder Finder is a searchable live database</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>rolling</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Varies by call. FCDO funds CSOs through mechanisms such as Aid Connect, which invites proposals from CSO consortia. Bond advises contacting FCDO country offices directly, as some funding is distributed at country level.</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>No open call matched to Give to Africa's programs at the time of this search. Listed as a channel to monitor rather than an opportunity - the Ghana Governance Programme shows FCDO does fund Ghanaian civil society.</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>https://devtracker.fcdo.gov.uk/countries/GH/projects/</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>NO SPECIFIC CALL. Search the FCDO Funder Finder and the UK government funding portal for live opportunities, and see Bond's funding page: https://www.bond.org.uk/resources-support/funding/ Bond specifically advises contacting the FCDO Ghana country office directly, since some funds are distributed at country level.</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bond.org.uk/resources-support/funding/</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>Add FCDO Funder Finder to the daily monitor's source rotation. Consider contacting the FCDO Ghana country office directly, which Bond specifically recommends for country-level funds.</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr">
+        <is>
+          <t>Mechanism and guidance confirmed; NO specific open opportunity found</t>
+        </is>
+      </c>
+      <c r="Q14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15" ht="96" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>2 - Open / rolling</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
           <t>UNDP / Green Climate Fund - Ghana Shea Landscape Emission Reductions Project (GSLERP) - RELATIONSHIP ONLY, no open call</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Multilateral (GCF / UNDP, delivered with the Global Shea Alliance)</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>NO OPEN CALL - implementing partners already selected</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Project total $54.5M. No open partner award - the 17 NGO implementing partner slots are filled.</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>No open call. The NGO call for proposals is archived - it dates from the project's 2020-21 startup.</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>NOT CURRENTLY OPEN. The original two-stage EOI (NGO submits to Global Shea Alliance, then pairs with a GSA private-sector member in a PPP including women's cooperatives) ran during project startup. GSLERP was approved by the GCF in 2020 for a seven-year run and is now in delivery with 17 NGO implementing partners and 5 seedling suppliers already engaged.</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Thematically the closest match found - Northern Savannah Zone, shea, women's cooperatives, climate. But there is no application route, so it is a relationship target, not a funding opportunity. The live angle is the surrounding ecosystem: Global Shea Alliance membership, the private-sector GSA members who co-fund PPPs, and the W+ Standard work GSLERP began in 2025 to quantify women's outcomes.</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>https://www.undp.org/ghana/projects/ghana-shea-landscape-emission-reductions-project</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>not publicly listed (EOI is submitted to the Global Shea Alliance - see globalshea.com for contacts)</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M13" s="7" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
         <is>
           <t>NO APPLICATION ROUTE - the call is archived and the 17 implementing partner slots are filled. Do not look for a portal. Engage the Global Shea Alliance (globalshea.com) as a member and ask whether partner intake reopens before the project ends around 2027.</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>https://www.undp.org/ghana/projects/ghana-shea-landscapes-emission-reductions-project-gslerp</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr">
+      <c r="O15" s="4" t="inlineStr">
         <is>
           <t>Do NOT look for an application portal - there isn't one. Instead join / engage the Global Shea Alliance as a member and get known to the GSA private-sector companies funding the PPPs. Ask GSA directly whether partner intake will reopen before the project closes (~2027) and what a successor project looks like. The W+ Standard adoption is also worth tracking - it is a credential Give to Africa's cooperatives could carry.</t>
         </is>
       </c>
-      <c r="P13" s="8" t="inlineStr">
+      <c r="P15" s="8" t="inlineStr">
         <is>
           <t>CORRECTED Jul 29, 2026. Previously listed as an open rolling EOI - that was wrong. The call for proposals is an undated archived page; project timeline (2020 approval, 7 years) and the 17 already-selected implementing partners confirm the window closed years ago.</t>
         </is>
       </c>
-      <c r="Q13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14" ht="96" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>3 - Calendar for next cycle</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Conservation, Food and Health Foundation (CFH)</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Private foundation (US)</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>OPEN - two cycles a year, concept application first</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>$25,000 - $50,000 per year; grants awarded for one or two years, year two contingent on progress</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Two concept-application cycles annually; grants awarded Jul 1 and Dec 1. Next concept deadline reported as mid-December - CONFIRM exact date on the funder's portal.</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>2026-12-15</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Non-profits, NGOs, CSOs, CBOs, universities and academic institutions. Work must be in low- and lower-middle-income countries in Africa, Asia, Latin America or the Middle East - Ghana qualifies. Does NOT fund businesses, government agencies, humanitarian aid organisations, other foundations or churches. Crucially, the requirement is on where the WORK happens, not where the applicant is registered, so Give to Africa appears eligible to apply DIRECTLY as a US 501(c)(3).</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>STRONGEST DIRECT-APPLY FIT FOUND. Their three focus areas map onto the Ghana programme almost line for line: Conservation (climate change mitigation, local capacity building - shea parklands), Food (sustainable agriculture, small-scale farmer support - shea processing and women's collectives), Health (environmental and occupational health - the PPE procurement for ~1,000 women). They fund pilot projects, new initiatives, training and technical assistance, which is exactly the design-stage facility's profile.</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>https://cfhfoundation.grantsmanagement08.com/</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M14" s="6" t="inlineStr">
-        <is>
-          <t>APPLY HERE: https://cfhfoundation.grantsmanagement08.com/?page_id=6 - online two-phase system. Stage 1 is a SHORT concept application; a limited number are invited to full proposal. Confirm the current cycle's concept deadline on the portal before writing.</t>
-        </is>
-      </c>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t>https://cfhfoundation.grantsmanagement08.com/?page_id=6</t>
-        </is>
-      </c>
-      <c r="O14" s="4" t="inlineStr">
-        <is>
-          <t>Highest-value new lead. Confirm the next concept deadline on their portal, then submit a concept for the PPE and occupational-health component or the shea parkland conservation angle - both are cleaner fits than the factory build, since CFH funds pilots and technical assistance rather than capital works.</t>
-        </is>
-      </c>
-      <c r="P14" s="4" t="inlineStr">
-        <is>
-          <t>Focus areas, grant size, eligibility categories, two-phase process and award dates confirmed across multiple sources. NEEDS VERIFICATION on the exact next concept deadline - sources give conflicting dates. Confirm on the portal.</t>
-        </is>
-      </c>
-      <c r="Q14" s="4" t="inlineStr">
+      <c r="Q15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16" ht="96" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>2 - Open / rolling</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Vons Foundation / Albertsons Companies Foundation - Southern California</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Corporate foundation (grocery retail)</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>OPEN - applications reviewed quarterly</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>$1,000 - $5,000 typical for a first-time funded organisation in Southern California</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Rolling - reviewed quarterly; allow at least 8 weeks for a decision</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>rolling</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>501(c)(3) serving communities where the company operates. Focus: K-12 education, hunger, public health, veterans. IMPORTANT: all California applications REQUIRE AN EMPLOYEE SPONSOR - typically a volunteer, board member, or someone your organisation has helped. If you have no employee in your network, the foundation explicitly suggests asking your LOCAL STORE MANAGER to sponsor you.</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Same category and same playbook as the confirmed Smart &amp; Final award. A California 501(c)(3) with a store-level relationship. Small money, quick cycle, and it builds the local corporate track record that makes larger California funders easier.</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>http://vonsfoundation.org</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t>APPLY HERE: http://vonsfoundation.org/get-funded/grant-application-process-southern-ca/ - online application. Guidelines: http://vonsfoundation.org/get-funded/grant-funding-guidelines-southern-ca/ Secure the employee sponsor BEFORE applying; the foundation contacts them directly before considering the application.</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>http://vonsfoundation.org/get-funded/grant-application-process-southern-ca/</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>Identify an employee sponsor first - ask the local Vons store manager, exactly as the foundation suggests. Then apply. Frame around hunger or public health, which are their stated priorities.</t>
+        </is>
+      </c>
+      <c r="P16" s="4" t="inlineStr">
+        <is>
+          <t>Grant range, quarterly review, employee-sponsor requirement and application URLs confirmed from the foundation's own site.</t>
+        </is>
+      </c>
+      <c r="Q16" s="4" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="96" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>3 - Calendar for next cycle</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>UN Women's Peace &amp; Humanitarian Fund (WPHF) - Rapid Response Window</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Multilateral (UN)</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Not published in the summary reviewed</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Concept notes accepted through Dec 31, 2026</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>International and regional NGOs partnering under the Rapid Response Window, in ODA-eligible countries with active peace processes.</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>WEAK fit. Ghana has no active peace process, so the window's core criterion is not met. Listed only for completeness on the multilateral side.</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>https://wphfund.org</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M15" s="4" t="inlineStr">
-        <is>
-          <t>CALLS ARE POSTED AT: https://wphfund.org - open calls appear there as they launch, each with its own submission instructions. No standing portal. Weak fit for Ghana regardless.</t>
-        </is>
-      </c>
-      <c r="N15" s="4" t="inlineStr">
-        <is>
-          <t>https://wphfund.org/call-for-proposals-for-rapid-response-window-i-rngo-partners/</t>
-        </is>
-      </c>
-      <c r="O15" s="4" t="inlineStr">
-        <is>
-          <t>Deprioritize unless Give to Africa adds programming in a conflict-affected country. Revisit only if the portfolio shifts.</t>
-        </is>
-      </c>
-      <c r="P15" s="4" t="inlineStr">
-        <is>
-          <t>Window and closing date confirmed; grant size not confirmed</t>
-        </is>
-      </c>
-      <c r="Q15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16" ht="96" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>3 - Calendar for next cycle</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>UNDP / GEF Small Grants Programme (SGP) Ghana</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Multilateral (UNDP / Global Environment Facility)</t>
-        </is>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>CLOSED - annual, reopens approx. Feb-Mar</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Up to $30,000 per initiative</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>2026 round closed Mar 13, 2026 (window ran Feb 23 - Mar 13). Expect a similar window in 2027.</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>2027-03-13</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Local Ghanaian NGOs/non-profits with valid Registrar General's Department and Social Welfare certificates, or CBOs / social enterprises recognized by the District Assembly and Ghana EPA. the Minerals Development Fund (MDF), Ghana would be the applicant; Give to Africa cannot apply directly.</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>EXCELLENT strategic fit. The 2026 priority geography was the Black Volta Basin - Wa-West (Upper West), Bole, Sawla-Tuna-Kalba and Central Gonja (Savannah Region) - which is the same northern Ghana shea-gathering belt the the Minerals Development Fund (MDF), Ghana partnership already works in. Focus areas include sustainable agriculture and community-based conservation.</t>
-        </is>
-      </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>https://www.undp.org/ghana</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed (proposal guidelines and template are posted with each call on the UNDP Ghana site)</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M16" s="7" t="inlineStr">
-        <is>
-          <t>NO OPEN CALL - the 2026 round closed Mar 13. Calls are posted on the UNDP Ghana site and the country page at https://sgp.undp.org (Ghana). CONTACT: the 2026 call published akosua.bireduaa.aninakwa@undp.org for enquiries - email to confirm the 2027 timetable. the Minerals Development Fund (MDF), Ghana must be the applicant and needs valid Registrar General + Social Welfare certificates.</t>
-        </is>
-      </c>
-      <c r="N16" s="4" t="inlineStr">
-        <is>
-          <t>https://www.undp.org/ghana/press-releases/2026-call-proposals-gef-small-grant-programme-ghana</t>
-        </is>
-      </c>
-      <c r="O16" s="4" t="inlineStr">
-        <is>
-          <t>Put a calendar reminder for early February 2027. Confirm now that the Minerals Development Fund (MDF), Ghana's Registrar General and Social Welfare certificates are current - that paperwork is the usual disqualifier, and it takes months to fix.</t>
-        </is>
-      </c>
-      <c r="P16" s="4" t="inlineStr">
-        <is>
-          <t>Amount, deadline, eligibility and priority districts confirmed across multiple listings</t>
-        </is>
-      </c>
-      <c r="Q16" s="4" t="inlineStr"/>
     </row>
     <row r="17" ht="96" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
@@ -1861,47 +1869,47 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>WACSI / Wilde Ganzen - Match Funding for Civil Society Organisations in Ghana</t>
+          <t>Conservation, Food and Health Foundation (CFH)</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Foundation (regional intermediary)</t>
+          <t>Private foundation (US)</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>CLOSED - annual, 2026 round closed Apr 27</t>
+          <t>OPEN - two cycles a year, concept application first</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Up to $5,000 in match funding, plus coaching and a small kick-start grant</t>
+          <t>$25,000 - $50,000 per year; grants awarded for one or two years, year two contingent on progress</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>2026 round closed Apr 27, 2026. Expect a similar spring window in 2027.</t>
+          <t>Two concept-application cycles annually; grants awarded Jul 1 and Dec 1. Next concept deadline reported as mid-December - CONFIRM exact date on the funder's portal.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>2027-04-27</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Civil society organisations in Ghana. Organisations must raise at least 50% of project funds LOCALLY - the fund matches up to 50%. Delivered with the Change the Game Academy, which focuses on local fundraising capacity.</t>
+          <t>Non-profits, NGOs, CSOs, CBOs, universities and academic institutions. Work must be in low- and lower-middle-income countries in Africa, Asia, Latin America or the Middle East - Ghana qualifies. Does NOT fund businesses, government agencies, humanitarian aid organisations, other foundations or churches. Crucially, the requirement is on where the WORK happens, not where the applicant is registered, so Give to Africa appears eligible to apply DIRECTLY as a US 501(c)(3).</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Small money, but unusually well aligned in method. The whole premise - mobilizing local resources and matching them - is what YENDAA does as a platform. A win here is a credible proof point for YENDAA's local-giving thesis, and the coaching component has standalone value for the fiscal sponsorship cohort.</t>
+          <t>STRONGEST DIRECT-APPLY FIT FOUND. Their three focus areas map onto the Ghana programme almost line for line: Conservation (climate change mitigation, local capacity building - shea parklands), Food (sustainable agriculture, small-scale farmer support - shea processing and women's collectives), Health (environmental and occupational health - the PPE procurement for ~1,000 women). They fund pilot projects, new initiatives, training and technical assistance, which is exactly the design-stage facility's profile.</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>https://wacsi.org</t>
+          <t>https://cfhfoundation.grantsmanagement08.com/</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
@@ -1914,27 +1922,31 @@
           <t>not publicly listed</t>
         </is>
       </c>
-      <c r="M17" s="7" t="inlineStr">
-        <is>
-          <t>NO OPEN CALL - the 2026 round closed Apr 27. CALL PAGE: https://wacsi.org/call-for-applications-match-funding-for-civil-society-organisations-in-ghana-2026/ The Terms of Reference and application form download from wacsi.org when a round is live. Ghana-registered CSOs only, and you must raise 50% locally first.</t>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>APPLY HERE: https://cfhfoundation.grantsmanagement08.com/?page_id=6 - online two-phase system. Stage 1 is a SHORT concept application; a limited number are invited to full proposal. Confirm the current cycle's concept deadline on the portal before writing.</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>https://wacsi.org/call-for-applications-match-funding-for-civil-society-organisations-in-ghana-2026/</t>
+          <t>https://cfhfoundation.grantsmanagement08.com/?page_id=6</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>Calendar for March 2027. Worth approaching WACSI now as a relationship rather than an applicant - they are a regional hub for exactly the West African CSOs YENDAA wants to list.</t>
+          <t>Highest-value new lead. Confirm the next concept deadline on their portal, then submit a concept for the PPE and occupational-health component or the shea parkland conservation angle - both are cleaner fits than the factory build, since CFH funds pilots and technical assistance rather than capital works.</t>
         </is>
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>Amount, match requirement, partners and deadline confirmed</t>
-        </is>
-      </c>
-      <c r="Q17" s="4" t="inlineStr"/>
+          <t>Focus areas, grant size, eligibility categories, two-phase process and award dates confirmed across multiple sources. NEEDS VERIFICATION on the exact next concept deadline - sources give conflicting dates. Confirm on the portal.</t>
+        </is>
+      </c>
+      <c r="Q17" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="96" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
@@ -1944,52 +1956,52 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Canada Fund for Local Initiatives (CFLI) - Ghana</t>
+          <t>UN Women's Peace &amp; Humanitarian Fund (WPHF) - Rapid Response Window</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Foreign government (Global Affairs Canada)</t>
+          <t>Multilateral (UN)</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>CLOSED - annual, reopens approx. Feb-Apr</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>CAD $25,000 - $45,000 average per project (CAD $200,000 total Ghana envelope)</t>
+          <t>Not published in the summary reviewed</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>2026 round closed May 10, 2026. Expect the 2027 call around Feb-Apr 2027.</t>
+          <t>Concept notes accepted through Dec 31, 2026</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>2027-04-30</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Broad and unusually favorable: local NGOs and non-profits, local academic institutions, AND international non-governmental organizations working on local development activities. Give to Africa appears eligible to apply directly.</t>
+          <t>International and regional NGOs partnering under the Rapid Response Window, in ODA-eligible countries with active peace processes.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>2026 Ghana themes were democratic governance / human rights and peace &amp; security, with gender equality as a cross-cutting theme. Themes rotate year to year - if a 2027 theme touches women's economic empowerment or climate, the the Minerals Development Fund (MDF), Ghana shea work fits cleanly.</t>
+          <t>WEAK fit. Ghana has no active peace process, so the window's core criterion is not met. Listed only for completeness on the multilateral side.</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>https://www.international.gc.ca/world-monde/funding-financement/cfli-fcil/ghana.aspx?lang=eng</t>
+          <t>https://wphfund.org</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>ghanacfli@international.gc.ca</t>
+          <t>not publicly listed</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -1997,24 +2009,24 @@
           <t>not publicly listed</t>
         </is>
       </c>
-      <c r="M18" s="7" t="inlineStr">
-        <is>
-          <t>NO OPEN CALL - 2026 round closed May 10. COUNTRY PAGE: https://www.international.gc.ca/world-monde/funding-financement/cfli-fcil/ghana.aspx?lang=eng When open, apply either through the Collaboration@International (C@I) portal - which needs a Government of Canada GCKey username first - or by emailing the completed application form and budget to ghanacfli@international.gc.ca. A gender-based analysis is mandatory. Email now to be notified for 2027.</t>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>CALLS ARE POSTED AT: https://wphfund.org - open calls appear there as they launch, each with its own submission instructions. No standing portal. Weak fit for Ghana regardless.</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>https://www.international.gc.ca/world-monde/funding-financement/cfli-fcil/ghana.aspx?lang=eng</t>
+          <t>https://wphfund.org/call-for-proposals-for-rapid-response-window-i-rngo-partners/</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>Email ghanacfli@international.gc.ca now to ask to be notified when the 2027 call opens, and ask what the 2027 thematic priorities will be. This is one of the few government funders on this list where Give to Africa can be the direct applicant.</t>
+          <t>Deprioritize unless Give to Africa adds programming in a conflict-affected country. Revisit only if the portfolio shifts.</t>
         </is>
       </c>
       <c r="P18" s="4" t="inlineStr">
         <is>
-          <t>Amounts, deadline, eligibility and contact email confirmed</t>
+          <t>Window and closing date confirmed; grant size not confirmed</t>
         </is>
       </c>
       <c r="Q18" s="4" t="inlineStr"/>
@@ -2027,80 +2039,84 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Investing for Employment (IFE) / Invest for Jobs - Ghana Call for Proposals</t>
+          <t>Smart &amp; Final Charitable Foundation</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Foreign government (German development bank KfW)</t>
+          <t>Corporate foundation (US retail)</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>CLOSED - annual, window ran Mar 20 - Jun 1 in 2026</t>
+          <t>PRIOR FUNDER - renew annually</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>EUR 800,000 - EUR 10,000,000 per project. Non-profit projects with no revenue generation are covered up to 90% of investment costs; non-profit with revenue generation up to 75%.</t>
+          <t>Not published; product and monetary donations</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>2026 window closed Jun 1, 2026 (17:00 CEST). Expect a similar Mar-Jun window in 2027.</t>
+          <t>Reported application deadline Jan 6, 2026 - passed</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>2027-06-01</t>
+          <t>2027-01-06</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Private companies as well as public and NON-PROFIT organisations. All projects must create jobs in the private sector. Two-stage: concept note via the SmartME portal first, full proposal by invitation.</t>
+          <t>501(c)(3) serving communities the company operates in - Arizona, California, Nevada. Focus: health and wellness, education, hunger relief, team sports and youth development, disaster relief. Give to Africa has qualified and been funded.</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>BEST NEW FIND. The the Minerals Development Fund (MDF), Ghana shea butter factories are a job-creation investment in exactly the country and sector IFE funds, and the 90% cost coverage for non-revenue non-profit projects is unusually generous. Scale is far above anything else on this list.</t>
+          <t>CONFIRMED FUNDER - Smart &amp; Final awarded Give to Africa a grant in 2025. Give to Africa is a California 501(c)(3) and qualified. This establishes the model for the whole California retail/corporate category: these funders give on the basis of the ORGANISATION being local, and a store-level or employee relationship matters more than programme geography.</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>https://invest-for-jobs.com/en/investing-for-employment</t>
+          <t>https://www.smartandfinal.com</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>cfp-ife.2026@invest-for-jobs.com (2026 cycle address - expect the year to change for 2027)</t>
+          <t>not publicly listed</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M19" s="7" t="inlineStr">
-        <is>
-          <t>NO OPEN GHANA CALL - the Ghana window closed Jun 1, 2026. A different window (Cote d'Ivoire, Egypt, Morocco) runs Apr 15 - Jun 30, 2026, which shows the cycle is live and rotating. ALL CALLS: https://invest-for-jobs.com/en/calls-for-proposals-overview Applications are submitted ONLY through the SmartME online platform - set up an account and watch the tutorials now: https://invest-for-jobs.com/en/introduction-to-smartme Stage 1 is a concept note scored on jobs created. Email cfp-ife.2026@invest-for-jobs.com to be notified.</t>
+          <t>323-869-7506 (published foundation contact)</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>PRIOR FUNDER - renew. Reported application deadline Jan 6 (annual). Contact the foundation on 323-869-7506 to confirm the current cycle and reference the previous award. A renewal request from a funded grantee is a different and much easier conversation than a cold application.</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>https://invest-for-jobs.com/en/call-for-proposals-march-april-2026</t>
+          <t>https://www.theshareway.com/grant/smart--08852-smart-final-charitable-foundation-donations</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>Email the CfP address now to ask to be notified when the 2027 window opens and to confirm whether a U.S. 501(c)(3) can apply directly or must partner with the Minerals Development Fund (MDF), Ghana. Start modelling the factory job-creation numbers - that is the metric IFE selects on.</t>
-        </is>
-      </c>
-      <c r="P19" s="4" t="inlineStr">
-        <is>
-          <t>Amounts, deadline, cost-coverage tiers, eligibility and contact email confirmed across KfW/GTAI/Invest-for-Jobs listings</t>
-        </is>
-      </c>
-      <c r="Q19" s="4" t="inlineStr"/>
+          <t>Diarise the January cycle and renew. Ask whoever handled last year's award who the internal contact was - that relationship is the asset, and it is also the template for approaching Vons, SDG&amp;E and the rest of the California corporate list.</t>
+        </is>
+      </c>
+      <c r="P19" s="8" t="inlineStr">
+        <is>
+          <t>CORRECTED Jul 30, 2026. Previously recorded as NOT ELIGIBLE on a reading of their published AZ/CA/NV geographic language. Victoria confirms Smart &amp; Final funded Give to Africa in 2025. An actual award overrides an inference from published guidelines - eligibility language describes where the company gives, not necessarily a restriction on where a local grantee's programmes operate.</t>
+        </is>
+      </c>
+      <c r="Q19" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="96" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
@@ -2110,52 +2126,52 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Common Fund for Commodities (CFC) - Annual Call for Proposals</t>
+          <t>UNDP / GEF Small Grants Programme (SGP) Ghana</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Multilateral (intergovernmental commodity body)</t>
+          <t>Multilateral (UNDP / Global Environment Facility)</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>CLOSED - 28th call closed Apr 1, 2026; watch for the 29th</t>
+          <t>CLOSED - annual, reopens approx. Feb-Mar</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Up to $1,500,000 (regular) / $300,000 (fast-track) - note: primarily LOANS and debt instruments, not pure grants</t>
+          <t>Up to $30,000 per initiative</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>28th call closed Apr 1, 2026</t>
+          <t>2026 round closed Mar 13, 2026 (window ran Feb 23 - Mar 13). Expect a similar window in 2027.</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>2027-03-13</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>SMEs, cooperatives, social enterprises, NGOs and public/private entities based or operating in one of 101 CFC member countries (Ghana is a member). Requires a minimum 3-year operating history and a financially viable project.</t>
+          <t>Local Ghanaian NGOs/non-profits with valid Registrar General's Department and Social Welfare certificates, or CBOs / social enterprises recognized by the District Assembly and Ghana EPA. the Minerals Development Fund (MDF), Ghana would be the applicant; Give to Africa cannot apply directly.</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Strong thematic fit for the shea value chain. CFC's stated priorities include local value addition, regenerative agriculture and women's entrepreneurship - the shea butter factory model hits all three. Be aware the instrument is mostly debt, so this suits the revenue-generating factory rather than grant-funded programming.</t>
+          <t>EXCELLENT strategic fit. The 2026 priority geography was the Black Volta Basin - Wa-West (Upper West), Bole, Sawla-Tuna-Kalba and Central Gonja (Savannah Region) - which is the same northern Ghana shea-gathering belt the the Minerals Development Fund (MDF), Ghana partnership already works in. Focus areas include sustainable agriculture and community-based conservation.</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>https://www.common-fund.org</t>
+          <t>https://www.undp.org/ghana</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>not publicly listed</t>
+          <t>not publicly listed (proposal guidelines and template are posted with each call on the UNDP Ghana site)</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
@@ -2163,24 +2179,24 @@
           <t>not publicly listed</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr">
-        <is>
-          <t>CALL PAGE: https://www.common-fund.org/call-for-proposals - the application form is downloadable there when a call is open. The 28th call closed Apr 1, 2026. Two-stage; English only; requires a 3-year operating track record. Mostly loans, not grants.</t>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>NO OPEN CALL - the 2026 round closed Mar 13. Calls are posted on the UNDP Ghana site and the country page at https://sgp.undp.org (Ghana). CONTACT: the 2026 call published akosua.bireduaa.aninakwa@undp.org for enquiries - email to confirm the 2027 timetable. the Minerals Development Fund (MDF), Ghana must be the applicant and needs valid Registrar General + Social Welfare certificates.</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>https://www.common-fund.org/call-for-proposals</t>
+          <t>https://www.undp.org/ghana/press-releases/2026-call-proposals-gef-small-grant-programme-ghana</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>Watch for the 29th call announcement. Before applying, decide whether the Minerals Development Fund (MDF), Ghana's factory model can service debt - if not, this is the wrong instrument regardless of fit.</t>
+          <t>Put a calendar reminder for early February 2027. Confirm now that the Minerals Development Fund (MDF), Ghana's Registrar General and Social Welfare certificates are current - that paperwork is the usual disqualifier, and it takes months to fix.</t>
         </is>
       </c>
       <c r="P20" s="4" t="inlineStr">
         <is>
-          <t>Amounts, deadline, eligibility and instrument type confirmed</t>
+          <t>Amount, deadline, eligibility and priority districts confirmed across multiple listings</t>
         </is>
       </c>
       <c r="Q20" s="4" t="inlineStr"/>
@@ -2193,47 +2209,47 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Dana Foundation - 2026 Grants Programme</t>
+          <t>WACSI / Wilde Ganzen - Match Funding for Civil Society Organisations in Ghana</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Foundation (regional intermediary)</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>NEEDS VERIFICATION - sources give conflicting deadlines</t>
+          <t>CLOSED - annual, 2026 round closed Apr 27</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>EUR 50,000 - EUR 150,000 per organization (sources differ)</t>
+          <t>Up to $5,000 in match funding, plus coaching and a small kick-start grant</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Conflicting: one source says May 5, 2026 (passed); another says Dec 31, 2026</t>
+          <t>2026 round closed Apr 27, 2026. Expect a similar spring window in 2027.</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>2027-04-27</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Locally led and governed organizations in low- or middle-income countries, generally with annual budgets under EUR 500,000, working across multiple dimensions of poverty at once.</t>
+          <t>Civil society organisations in Ghana. Organisations must raise at least 50% of project funds LOCALLY - the fund matches up to 50%. Delivered with the Change the Game Academy, which focuses on local fundraising capacity.</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit. 'Locally led and governed' may exclude a U.S.-headquartered 501(c)(3) - but it is a strong fit for the African organizations in the fiscal sponsorship cohort, which is itself a pitchable angle.</t>
+          <t>Small money, but unusually well aligned in method. The whole premise - mobilizing local resources and matching them - is what YENDAA does as a platform. A win here is a credible proof point for YENDAA's local-giving thesis, and the coaching component has standalone value for the fiscal sponsorship cohort.</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>https://wacsi.org</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
@@ -2248,22 +2264,22 @@
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>NO VERIFIED APPLICATION URL FOUND. This entry came from an aggregator roundup and the funder's own grants page could not be confirmed. Do not spend time on it until you verify the funder, the real deadline, and whether a US-based sponsor is eligible.</t>
+          <t>NO OPEN CALL - the 2026 round closed Apr 27. CALL PAGE: https://wacsi.org/call-for-applications-match-funding-for-civil-society-organisations-in-ghana-2026/ The Terms of Reference and application form download from wacsi.org when a round is live. Ghana-registered CSOs only, and you must raise 50% locally first.</t>
         </is>
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>https://africanngos.org/2026/06/09/african-ngo-funding-opportunities-june-july-2026/</t>
+          <t>https://wacsi.org/call-for-applications-match-funding-for-civil-society-organisations-in-ghana-2026/</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>Verify the real deadline and whether a U.S.-based sponsor is eligible before investing effort. If only locally led orgs qualify, redirect this to fiscal sponsorship cohort members.</t>
-        </is>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>NEEDS VERIFICATION - deadline and grant size both inconsistent across sources; funder's own site not confirmed</t>
+          <t>Calendar for March 2027. Worth approaching WACSI now as a relationship rather than an applicant - they are a regional hub for exactly the West African CSOs YENDAA wants to list.</t>
+        </is>
+      </c>
+      <c r="P21" s="4" t="inlineStr">
+        <is>
+          <t>Amount, match requirement, partners and deadline confirmed</t>
         </is>
       </c>
       <c r="Q21" s="4" t="inlineStr"/>
@@ -2276,52 +2292,52 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>U.S. African Development Foundation (USADF)</t>
+          <t>Canada Fund for Local Initiatives (CFLI) - Ghana</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>U.S. Government (independent federal agency)</t>
+          <t>Foreign government (Global Affairs Canada)</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>NOT ACCEPTING APPLICATIONS - per USADF's own apply page</t>
+          <t>CLOSED - annual, reopens approx. Feb-Apr</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Up to $250,000</t>
+          <t>CAD $25,000 - $45,000 average per project (CAD $200,000 total Ghana envelope)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Varies by country call - check usadf.gov for the current Ghana call</t>
+          <t>2026 round closed May 10, 2026. Expect the 2027 call around Feb-Apr 2027.</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>2027-04-30</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Applicant must be a 100% African-owned enterprise, cooperative, producer group or processor in an eligible country. Give to Africa is NOT directly eligible - the shea cooperative or the Minerals Development Fund (MDF), Ghana would be the grantee, with Give to Africa providing proposal and compliance support.</t>
+          <t>Broad and unusually favorable: local NGOs and non-profits, local academic institutions, AND international non-governmental organizations working on local development activities. Give to Africa appears eligible to apply directly.</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Strong on-mission fit - USADF funds exactly this kind of agricultural processor and women's producer group - but there is nothing to apply to at present.</t>
+          <t>2026 Ghana themes were democratic governance / human rights and peace &amp; security, with gender equality as a cross-cutting theme. Themes rotate year to year - if a 2027 theme touches women's economic empowerment or climate, the the Minerals Development Fund (MDF), Ghana shea work fits cleanly.</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>https://usadf.gov</t>
+          <t>https://www.international.gc.ca/world-monde/funding-financement/cfli-fcil/ghana.aspx?lang=eng</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>not publicly listed (each country call names its own submission address)</t>
+          <t>ghanacfli@international.gc.ca</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
@@ -2329,24 +2345,24 @@
           <t>not publicly listed</t>
         </is>
       </c>
-      <c r="M22" s="6" t="inlineStr">
-        <is>
-          <t>APPLY PAGE: https://www.usadf.gov/apply - but that page currently states applications are NOT being accepted. There is no open Ghana call to apply to right now. Check the page periodically; when a country call opens it names its own submission email address.</t>
+      <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t>NO OPEN CALL - 2026 round closed May 10. COUNTRY PAGE: https://www.international.gc.ca/world-monde/funding-financement/cfli-fcil/ghana.aspx?lang=eng When open, apply either through the Collaboration@International (C@I) portal - which needs a Government of Canada GCKey username first - or by emailing the completed application form and budget to ghanacfli@international.gc.ca. A gender-based analysis is mandatory. Email now to be notified for 2027.</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>https://usadf.gov/resources</t>
+          <t>https://www.international.gc.ca/world-monde/funding-financement/cfli-fcil/ghana.aspx?lang=eng</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>Confirm whether Ghana is in the current eligible-country list, then position the shea cooperative as applicant. Even at partner-support level this is the largest realistic U.S. government award on this list.</t>
-        </is>
-      </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>CORRECTED Jul 29, 2026. Previously listed as open with periodic country calls. USADF's own apply page states applications are not being accepted at this time. Ghana eligibility also remains unconfirmed - sources conflict.</t>
+          <t>Email ghanacfli@international.gc.ca now to ask to be notified when the 2027 call opens, and ask what the 2027 thematic priorities will be. This is one of the few government funders on this list where Give to Africa can be the direct applicant.</t>
+        </is>
+      </c>
+      <c r="P22" s="4" t="inlineStr">
+        <is>
+          <t>Amounts, deadline, eligibility and contact email confirmed</t>
         </is>
       </c>
       <c r="Q22" s="4" t="inlineStr"/>
@@ -2359,416 +2375,412 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
+          <t>Investing for Employment (IFE) / Invest for Jobs - Ghana Call for Proposals</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Foreign government (German development bank KfW)</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED - annual, window ran Mar 20 - Jun 1 in 2026</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>EUR 800,000 - EUR 10,000,000 per project. Non-profit projects with no revenue generation are covered up to 90% of investment costs; non-profit with revenue generation up to 75%.</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>2026 window closed Jun 1, 2026 (17:00 CEST). Expect a similar Mar-Jun window in 2027.</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>2027-06-01</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Private companies as well as public and NON-PROFIT organisations. All projects must create jobs in the private sector. Two-stage: concept note via the SmartME portal first, full proposal by invitation.</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>BEST NEW FIND. The the Minerals Development Fund (MDF), Ghana shea butter factories are a job-creation investment in exactly the country and sector IFE funds, and the 90% cost coverage for non-revenue non-profit projects is unusually generous. Scale is far above anything else on this list.</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>https://invest-for-jobs.com/en/investing-for-employment</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>cfp-ife.2026@invest-for-jobs.com (2026 cycle address - expect the year to change for 2027)</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>NO OPEN GHANA CALL - the Ghana window closed Jun 1, 2026. A different window (Cote d'Ivoire, Egypt, Morocco) runs Apr 15 - Jun 30, 2026, which shows the cycle is live and rotating. ALL CALLS: https://invest-for-jobs.com/en/calls-for-proposals-overview Applications are submitted ONLY through the SmartME online platform - set up an account and watch the tutorials now: https://invest-for-jobs.com/en/introduction-to-smartme Stage 1 is a concept note scored on jobs created. Email cfp-ife.2026@invest-for-jobs.com to be notified.</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>https://invest-for-jobs.com/en/call-for-proposals-march-april-2026</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>Email the CfP address now to ask to be notified when the 2027 window opens and to confirm whether a U.S. 501(c)(3) can apply directly or must partner with the Minerals Development Fund (MDF), Ghana. Start modelling the factory job-creation numbers - that is the metric IFE selects on.</t>
+        </is>
+      </c>
+      <c r="P23" s="4" t="inlineStr">
+        <is>
+          <t>Amounts, deadline, cost-coverage tiers, eligibility and contact email confirmed across KfW/GTAI/Invest-for-Jobs listings</t>
+        </is>
+      </c>
+      <c r="Q23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24" ht="96" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>3 - Calendar for next cycle</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Common Fund for Commodities (CFC) - Annual Call for Proposals</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Multilateral (intergovernmental commodity body)</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED - 28th call closed Apr 1, 2026; watch for the 29th</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Up to $1,500,000 (regular) / $300,000 (fast-track) - note: primarily LOANS and debt instruments, not pure grants</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>28th call closed Apr 1, 2026</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>SMEs, cooperatives, social enterprises, NGOs and public/private entities based or operating in one of 101 CFC member countries (Ghana is a member). Requires a minimum 3-year operating history and a financially viable project.</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Strong thematic fit for the shea value chain. CFC's stated priorities include local value addition, regenerative agriculture and women's entrepreneurship - the shea butter factory model hits all three. Be aware the instrument is mostly debt, so this suits the revenue-generating factory rather than grant-funded programming.</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.common-fund.org</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>CALL PAGE: https://www.common-fund.org/call-for-proposals - the application form is downloadable there when a call is open. The 28th call closed Apr 1, 2026. Two-stage; English only; requires a 3-year operating track record. Mostly loans, not grants.</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.common-fund.org/call-for-proposals</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>Watch for the 29th call announcement. Before applying, decide whether the Minerals Development Fund (MDF), Ghana's factory model can service debt - if not, this is the wrong instrument regardless of fit.</t>
+        </is>
+      </c>
+      <c r="P24" s="4" t="inlineStr">
+        <is>
+          <t>Amounts, deadline, eligibility and instrument type confirmed</t>
+        </is>
+      </c>
+      <c r="Q24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25" ht="96" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>3 - Calendar for next cycle</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Dana Foundation - 2026 Grants Programme</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION - sources give conflicting deadlines</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>EUR 50,000 - EUR 150,000 per organization (sources differ)</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Conflicting: one source says May 5, 2026 (passed); another says Dec 31, 2026</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Locally led and governed organizations in low- or middle-income countries, generally with annual budgets under EUR 500,000, working across multiple dimensions of poverty at once.</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Moderate fit. 'Locally led and governed' may exclude a U.S.-headquartered 501(c)(3) - but it is a strong fit for the African organizations in the fiscal sponsorship cohort, which is itself a pitchable angle.</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="inlineStr">
+        <is>
+          <t>NO VERIFIED APPLICATION URL FOUND. This entry came from an aggregator roundup and the funder's own grants page could not be confirmed. Do not spend time on it until you verify the funder, the real deadline, and whether a US-based sponsor is eligible.</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>https://africanngos.org/2026/06/09/african-ngo-funding-opportunities-june-july-2026/</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>Verify the real deadline and whether a U.S.-based sponsor is eligible before investing effort. If only locally led orgs qualify, redirect this to fiscal sponsorship cohort members.</t>
+        </is>
+      </c>
+      <c r="P25" s="8" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION - deadline and grant size both inconsistent across sources; funder's own site not confirmed</t>
+        </is>
+      </c>
+      <c r="Q25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26" ht="96" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>3 - Calendar for next cycle</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>U.S. African Development Foundation (USADF)</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>U.S. Government (independent federal agency)</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>NOT ACCEPTING APPLICATIONS - per USADF's own apply page</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Up to $250,000</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Varies by country call - check usadf.gov for the current Ghana call</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Applicant must be a 100% African-owned enterprise, cooperative, producer group or processor in an eligible country. Give to Africa is NOT directly eligible - the shea cooperative or the Minerals Development Fund (MDF), Ghana would be the grantee, with Give to Africa providing proposal and compliance support.</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>Strong on-mission fit - USADF funds exactly this kind of agricultural processor and women's producer group - but there is nothing to apply to at present.</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>https://usadf.gov</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed (each country call names its own submission address)</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M26" s="6" t="inlineStr">
+        <is>
+          <t>APPLY PAGE: https://www.usadf.gov/apply - but that page currently states applications are NOT being accepted. There is no open Ghana call to apply to right now. Check the page periodically; when a country call opens it names its own submission email address.</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>https://usadf.gov/resources</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>Confirm whether Ghana is in the current eligible-country list, then position the shea cooperative as applicant. Even at partner-support level this is the largest realistic U.S. government award on this list.</t>
+        </is>
+      </c>
+      <c r="P26" s="8" t="inlineStr">
+        <is>
+          <t>CORRECTED Jul 29, 2026. Previously listed as open with periodic country calls. USADF's own apply page states applications are not being accepted at this time. Ghana eligibility also remains unconfirmed - sources conflict.</t>
+        </is>
+      </c>
+      <c r="Q26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27" ht="96" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>3 - Calendar for next cycle</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
           <t>United Nations Democracy Fund (UNDEF)</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Multilateral (UN)</t>
         </is>
       </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>CLOSED - annual window, 2026 round not yet announced</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>Up to $300,000 per project (two-year projects)</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>Annual window, historically about a month long (a recent round ran Nov 1-30)</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>Civil society organizations and NGOs promoting democracy; preference for countries in democratic transition and consolidation, least developed countries, and low/middle-income countries.</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>Moderate fit. Would need to be framed around civil-society strengthening - the fiscal sponsorship program and YENDAA's transparency/verification infrastructure for African-led organizations is the most credible angle.</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="J27" s="4" t="inlineStr">
         <is>
           <t>https://www.un.org/democracyfund/en</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M23" s="6" t="inlineStr">
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M27" s="6" t="inlineStr">
         <is>
           <t>APPLY VIA THE OPPS PORTAL: https://www.un.org/democracyfund/en/content/how-apply-online-project-proposal-system-opps You must REGISTER YOUR ORGANIZATION FIRST to receive a login - do that before the window opens, since the window is short (historically about a month, often November). Technical support: undefproposal@un.org. Draft offline using their blank proposal form, then paste in.</t>
         </is>
       </c>
-      <c r="N23" s="4" t="inlineStr">
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>https://www.un.org/democracyfund/en/apply-for-funding</t>
         </is>
       </c>
-      <c r="O23" s="4" t="inlineStr">
+      <c r="O27" s="4" t="inlineStr">
         <is>
           <t>Check the UNDEF site monthly from October onward. The window is short and there is no extension, so a draft concept must exist before it opens.</t>
         </is>
       </c>
-      <c r="P23" s="4" t="inlineStr">
+      <c r="P27" s="4" t="inlineStr">
         <is>
           <t>Grant ceiling and eligibility confirmed; 2026 round dates not yet published</t>
         </is>
       </c>
-      <c r="Q23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24" ht="96" customHeight="1">
-      <c r="A24" s="13" t="inlineStr">
-        <is>
-          <t>4 - Low priority</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>USDA Foreign Agricultural Service - McGovern-Dole International Food for Education FY2026</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>U.S. Government (federal)</t>
-        </is>
-      </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>CLOSED for FY2026</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Not published in the summary reviewed (multi-million, multi-year)</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Closed Jun 22, 2026</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Non-profits, cooperatives, universities and similar entities. Non-priority countries are accepted but rarely funded.</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>Poor fit. FY2026 priority countries in West Africa were Guinea (Conakry) and Liberia - not Ghana. Education focus is school feeding and child nutrition, not workforce development.</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>https://www.fas.usda.gov</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M24" s="7" t="inlineStr">
-        <is>
-          <t>CLOSED for FY2026. Future rounds post on grants.gov and at fas.usda.gov. Ghana is not a priority country - watch the FY2027 priority-country announcement before investing any time.</t>
-        </is>
-      </c>
-      <c r="N24" s="4" t="inlineStr">
-        <is>
-          <t>https://www.fas.usda.gov/newsroom/stakeholder-notice-usda-publishes-fy-2026-notice-funding-opportunity-mcgovern-dole-program</t>
-        </is>
-      </c>
-      <c r="O24" s="4" t="inlineStr">
-        <is>
-          <t>Skip. Listed so the FY2027 priority-country announcement can be checked - if Ghana is added, reassess.</t>
-        </is>
-      </c>
-      <c r="P24" s="4" t="inlineStr">
-        <is>
-          <t>Deadline and priority countries confirmed</t>
-        </is>
-      </c>
-      <c r="Q24" s="4" t="inlineStr"/>
-    </row>
-    <row r="25" ht="96" customHeight="1">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>4 - Low priority</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>USDA Foreign Agricultural Service - Food for Progress FY2026</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>U.S. Government (federal)</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>CLOSED for FY2026</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>$28,000,000 - $35,000,000 per award (up to $226M total)</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>Closed Jul 6, 2026</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>Governments, intergovernmental organizations, PVOs, non-profit agricultural organizations and cooperatives, NGOs, universities, and other private entities. Award sizes require major institutional capacity.</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>Poor fit at current scale. FY2026 priority countries were Bangladesh, Bolivia, Ecuador, Morocco, the Philippines, Sri Lanka and Thailand - Ghana was not among them.</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>https://www.fas.usda.gov/programs/food-progress</t>
-        </is>
-      </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M25" s="7" t="inlineStr">
-        <is>
-          <t>CLOSED for FY2026. Future rounds post on grants.gov and at https://www.fas.usda.gov/programs/food-progress - not viable at your current scale regardless.</t>
-        </is>
-      </c>
-      <c r="N25" s="4" t="inlineStr">
-        <is>
-          <t>https://www.fas.usda.gov/newsroom/usda-publishes-fy-2026-notices-funding-opportunity-food-progress</t>
-        </is>
-      </c>
-      <c r="O25" s="4" t="inlineStr">
-        <is>
-          <t>Not viable now - award sizes are far above Give to Africa's current capacity and Ghana is off the priority list. Revisit only as a sub-awardee to a large prime.</t>
-        </is>
-      </c>
-      <c r="P25" s="4" t="inlineStr">
-        <is>
-          <t>Amounts, deadline and priority countries confirmed</t>
-        </is>
-      </c>
-      <c r="Q25" s="4" t="inlineStr"/>
-    </row>
-    <row r="26" ht="96" customHeight="1">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t>4 - Low priority</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>UN Women - Spotlight Initiative Africa Regional Programme (SIARP) 2.0</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Multilateral (UN)</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="inlineStr">
-        <is>
-          <t>CLOSED - deadline passed Jul 27, 2026</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>$110,000 - $548,000 (27-month projects, Oct 2026 - Dec 2028)</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>Jul 27, 2026, 5pm East Africa Time</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>CSOs, women's rights organizations, coalitions and networks operating at continental, regional, sub-regional or multi-country level in Africa, with demonstrated gender-equality programming experience.</t>
-        </is>
-      </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>Would have been a good multi-country fit given the cross-border structure, but the thematic focus (ending violence against women and girls, SRHR, survivor services) sits outside Give to Africa's four programs.</t>
-        </is>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>https://africa.unwomen.org</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M26" s="7" t="inlineStr">
-        <is>
-          <t>CLOSED - deadline passed Jul 27, 2026. Future UN Women Africa calls are posted at https://africa.unwomen.org under programme implementation.</t>
-        </is>
-      </c>
-      <c r="N26" s="4" t="inlineStr">
-        <is>
-          <t>https://africa.unwomen.org/en/programme-implementation/2026/06/call-for-proposals-for-civil-society-partnerships-for-implementation-of-the-spotlight-initiative-africa-regional-programme-siarp-20</t>
-        </is>
-      </c>
-      <c r="O26" s="4" t="inlineStr">
-        <is>
-          <t>Missed for this cycle. Worth tracking UN Women Africa's calls generally - the multi-country eligibility structure suits Give to Africa's cross-border model better than most funders'.</t>
-        </is>
-      </c>
-      <c r="P26" s="4" t="inlineStr">
-        <is>
-          <t>Amounts, deadline and eligibility confirmed</t>
-        </is>
-      </c>
-      <c r="Q26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27" ht="96" customHeight="1">
-      <c r="A27" s="13" t="inlineStr">
-        <is>
-          <t>4 - Low priority</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Smart &amp; Final Charitable Foundation</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Corporate foundation (US retail)</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>NOT ELIGIBLE - geographic mismatch</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>Not published; product and monetary donations</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Reported application deadline Jan 6, 2026 - passed</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>2027-01-06</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>Supports nonprofits improving quality of life in communities the COMPANY SERVES - Arizona, California and Nevada. Focus areas: health and wellness, education, hunger relief, team sports and youth development, disaster relief. 501(c)(3) required.</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>NOT A FIT as things stand. Give to Africa is San Diego-registered, but the funded WORK must benefit AZ/CA/NV communities and all four Give to Africa programs operate in Africa. This would only become viable if Give to Africa ran a San Diego-facing program - diaspora engagement, local youth education, volunteer programming.</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>https://www.smartandfinal.com</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>323-869-7506 (published foundation contact)</t>
-        </is>
-      </c>
-      <c r="M27" s="4" t="inlineStr">
-        <is>
-          <t>NOT ELIGIBLE for current programming - do not apply. Their giving is restricted to communities the company serves in Arizona, California and Nevada.</t>
-        </is>
-      </c>
-      <c r="N27" s="4" t="inlineStr">
-        <is>
-          <t>https://www.theshareway.com/grant/smart--08852-smart-final-charitable-foundation-donations</t>
-        </is>
-      </c>
-      <c r="O27" s="4" t="inlineStr">
-        <is>
-          <t>Do not apply for Africa programming. Recorded so this ground is not re-searched. Revisit only if Give to Africa launches a San Diego-based program - see the note on local corporate funders in the method sheet.</t>
-        </is>
-      </c>
-      <c r="P27" s="4" t="inlineStr">
-        <is>
-          <t>Geographic restriction, focus areas and phone number confirmed. Deadline reported as Jan 6, 2026 and presumed annual.</t>
-        </is>
-      </c>
-      <c r="Q27" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
+      <c r="Q27" s="4" t="inlineStr"/>
     </row>
     <row r="28" ht="96" customHeight="1">
       <c r="A28" s="13" t="inlineStr">
@@ -2778,83 +2790,332 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
+          <t>USDA Foreign Agricultural Service - McGovern-Dole International Food for Education FY2026</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>U.S. Government (federal)</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>CLOSED for FY2026</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Not published in the summary reviewed (multi-million, multi-year)</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Closed Jun 22, 2026</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Non-profits, cooperatives, universities and similar entities. Non-priority countries are accepted but rarely funded.</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>Poor fit. FY2026 priority countries in West Africa were Guinea (Conakry) and Liberia - not Ghana. Education focus is school feeding and child nutrition, not workforce development.</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>https://www.fas.usda.gov</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M28" s="7" t="inlineStr">
+        <is>
+          <t>CLOSED for FY2026. Future rounds post on grants.gov and at fas.usda.gov. Ghana is not a priority country - watch the FY2027 priority-country announcement before investing any time.</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>https://www.fas.usda.gov/newsroom/stakeholder-notice-usda-publishes-fy-2026-notice-funding-opportunity-mcgovern-dole-program</t>
+        </is>
+      </c>
+      <c r="O28" s="4" t="inlineStr">
+        <is>
+          <t>Skip. Listed so the FY2027 priority-country announcement can be checked - if Ghana is added, reassess.</t>
+        </is>
+      </c>
+      <c r="P28" s="4" t="inlineStr">
+        <is>
+          <t>Deadline and priority countries confirmed</t>
+        </is>
+      </c>
+      <c r="Q28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29" ht="96" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>4 - Low priority</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>USDA Foreign Agricultural Service - Food for Progress FY2026</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>U.S. Government (federal)</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>CLOSED for FY2026</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>$28,000,000 - $35,000,000 per award (up to $226M total)</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Closed Jul 6, 2026</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Governments, intergovernmental organizations, PVOs, non-profit agricultural organizations and cooperatives, NGOs, universities, and other private entities. Award sizes require major institutional capacity.</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>Poor fit at current scale. FY2026 priority countries were Bangladesh, Bolivia, Ecuador, Morocco, the Philippines, Sri Lanka and Thailand - Ghana was not among them.</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.fas.usda.gov/programs/food-progress</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t>CLOSED for FY2026. Future rounds post on grants.gov and at https://www.fas.usda.gov/programs/food-progress - not viable at your current scale regardless.</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.fas.usda.gov/newsroom/usda-publishes-fy-2026-notices-funding-opportunity-food-progress</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t>Not viable now - award sizes are far above Give to Africa's current capacity and Ghana is off the priority list. Revisit only as a sub-awardee to a large prime.</t>
+        </is>
+      </c>
+      <c r="P29" s="4" t="inlineStr">
+        <is>
+          <t>Amounts, deadline and priority countries confirmed</t>
+        </is>
+      </c>
+      <c r="Q29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30" ht="96" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>4 - Low priority</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>UN Women - Spotlight Initiative Africa Regional Programme (SIARP) 2.0</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Multilateral (UN)</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>CLOSED - deadline passed Jul 27, 2026</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>$110,000 - $548,000 (27-month projects, Oct 2026 - Dec 2028)</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Jul 27, 2026, 5pm East Africa Time</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>CSOs, women's rights organizations, coalitions and networks operating at continental, regional, sub-regional or multi-country level in Africa, with demonstrated gender-equality programming experience.</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>Would have been a good multi-country fit given the cross-border structure, but the thematic focus (ending violence against women and girls, SRHR, survivor services) sits outside Give to Africa's four programs.</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>https://africa.unwomen.org</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M30" s="7" t="inlineStr">
+        <is>
+          <t>CLOSED - deadline passed Jul 27, 2026. Future UN Women Africa calls are posted at https://africa.unwomen.org under programme implementation.</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>https://africa.unwomen.org/en/programme-implementation/2026/06/call-for-proposals-for-civil-society-partnerships-for-implementation-of-the-spotlight-initiative-africa-regional-programme-siarp-20</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t>Missed for this cycle. Worth tracking UN Women Africa's calls generally - the multi-country eligibility structure suits Give to Africa's cross-border model better than most funders'.</t>
+        </is>
+      </c>
+      <c r="P30" s="4" t="inlineStr">
+        <is>
+          <t>Amounts, deadline and eligibility confirmed</t>
+        </is>
+      </c>
+      <c r="Q30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31" ht="96" customHeight="1">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>4 - Low priority</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
           <t>Segal Family Foundation</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="D31" s="14" t="inlineStr">
         <is>
           <t>NOT OPEN - invitation only</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>$10,000 - $100,000+ (averaging approx. $50,000; approx. $15M granted annually)</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>No deadline - does not accept unsolicited applications</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>Grassroots African-led organizations in education, youth empowerment and social entrepreneurship. Grantees come through referral only.</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>Very strong mission fit (trust-based philanthropy for African-led organizations) but there is no application route. This is a relationship-building target, not a proposal target.</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="J31" s="4" t="inlineStr">
         <is>
           <t>https://www.segalfamilyfoundation.org</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>not publicly listed</t>
-        </is>
-      </c>
-      <c r="M28" s="7" t="inlineStr">
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>not publicly listed</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="inlineStr">
         <is>
           <t>NO APPLICATION ROUTE - Segal does not accept unsolicited applications and works purely by referral. Do not submit anything. Map who in your network can make a warm introduction.</t>
         </is>
       </c>
-      <c r="N28" s="4" t="inlineStr">
+      <c r="N31" s="4" t="inlineStr">
         <is>
           <t>https://www.segalfamilyfoundation.org/what-we-do/invest/grantmaking/</t>
         </is>
       </c>
-      <c r="O28" s="4" t="inlineStr">
+      <c r="O31" s="4" t="inlineStr">
         <is>
           <t>Do not submit a proposal - it will not be read. Instead, map who in Give to Africa's network already holds a Segal relationship and pursue a warm referral. Their African-led portfolio overlaps heavily with YENDAA's target causes.</t>
         </is>
       </c>
-      <c r="P28" s="4" t="inlineStr">
+      <c r="P31" s="4" t="inlineStr">
         <is>
           <t>Referral-only model and grant range confirmed</t>
         </is>
       </c>
-      <c r="Q28" s="4" t="inlineStr"/>
+      <c r="Q31" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:Q28"/>
+  <autoFilter ref="A2:Q31"/>
   <mergeCells count="1">
     <mergeCell ref="A1:Q1"/>
   </mergeCells>
@@ -3015,7 +3276,7 @@
         </is>
       </c>
       <c r="B20" s="22" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21">
@@ -3035,7 +3296,7 @@
         </is>
       </c>
       <c r="B22" s="23" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23">
@@ -3045,7 +3306,7 @@
         </is>
       </c>
       <c r="B23" s="23" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24">
@@ -3055,7 +3316,7 @@
         </is>
       </c>
       <c r="B24" s="23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">

</xml_diff>